<commit_message>
update: deuda interna — 161 new rows, total 4.20B USD (Jun 2026)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 02-Jun-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 11-Jun-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,34 +845,34 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1733956076.73</v>
+        <v>1751774360.969999</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>530139315.8800001</v>
+        <v>536138968.9900001</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1161832928.36</v>
+        <v>1170652109.64</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>20685165.52</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>21298666.97</v>
+        <v>24298116.82</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>30.57397606517053</v>
+        <v>30.60548098746731</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>67.00474965611905</v>
+        <v>66.82664935179103</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>1.192946338006978</v>
+        <v>1.180812208516748</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.228327940703454</v>
+        <v>1.387057452224929</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.385658914728682</v>
+        <v>7.421304347826086</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4182598919.599999</v>
+        <v>4200417203.839999</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -2325,19 +2325,19 @@
         </is>
       </c>
       <c r="C57" s="9" t="n">
-        <v>9999429.58</v>
+        <v>27817713.82</v>
       </c>
       <c r="D57" s="9" t="n">
-        <v>9999429.58</v>
+        <v>15999082.69</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>0</v>
+        <v>8819181.280000001</v>
       </c>
       <c r="F57" s="9" t="n">
         <v>0</v>
       </c>
       <c r="G57" s="9" t="n">
-        <v>0</v>
+        <v>2999449.85</v>
       </c>
     </row>
   </sheetData>
@@ -3828,7 +3828,7 @@
         <v>8.0503</v>
       </c>
       <c r="E67" s="11" t="n">
-        <v>8.6188</v>
+        <v>8.6195</v>
       </c>
       <c r="F67" s="11" t="n">
         <v>9.0306</v>
@@ -3844,16 +3844,16 @@
         </is>
       </c>
       <c r="C68" s="7" t="n">
-        <v>6.8333</v>
+        <v>6.75</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>8.145799999999999</v>
+        <v>8.1073</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>8.809200000000001</v>
+        <v>8.7117</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>9.7354</v>
+        <v>9.382999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3870,7 +3870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1094"/>
+  <dimension ref="A1:N1112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -62912,6 +62912,978 @@
         </is>
       </c>
     </row>
+    <row r="1095">
+      <c r="A1095" s="19" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B1095" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1095" s="20" t="n">
+        <v>1018</v>
+      </c>
+      <c r="D1095" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1095" s="21" t="n">
+        <v>99.981796</v>
+      </c>
+      <c r="F1095" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1095" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1095" s="22" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1095" s="22" t="n">
+        <v>999817.96</v>
+      </c>
+      <c r="J1095" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1095" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1095" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1095" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1095" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="23" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B1096" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1096" s="24" t="n">
+        <v>984</v>
+      </c>
+      <c r="D1096" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1096" s="25" t="n">
+        <v>99.979884</v>
+      </c>
+      <c r="F1096" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1096" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1096" s="26" t="n">
+        <v>107650</v>
+      </c>
+      <c r="I1096" s="26" t="n">
+        <v>107628.35</v>
+      </c>
+      <c r="J1096" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1096" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1096" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1096" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1096" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="19" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B1097" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1097" s="20" t="n">
+        <v>984</v>
+      </c>
+      <c r="D1097" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1097" s="21" t="n">
+        <v>99.979884</v>
+      </c>
+      <c r="F1097" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1097" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1097" s="22" t="n">
+        <v>107650</v>
+      </c>
+      <c r="I1097" s="22" t="n">
+        <v>107628.35</v>
+      </c>
+      <c r="J1097" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1097" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1097" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1097" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1097" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="23" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B1098" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1098" s="24" t="n">
+        <v>984</v>
+      </c>
+      <c r="D1098" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1098" s="25" t="n">
+        <v>99.979884</v>
+      </c>
+      <c r="F1098" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1098" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1098" s="26" t="n">
+        <v>59000</v>
+      </c>
+      <c r="I1098" s="26" t="n">
+        <v>58988.13</v>
+      </c>
+      <c r="J1098" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1098" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1098" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1098" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1098" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="19" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B1099" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1099" s="20" t="n">
+        <v>294</v>
+      </c>
+      <c r="D1099" s="15" t="inlineStr">
+        <is>
+          <t>Hasta 1</t>
+        </is>
+      </c>
+      <c r="E1099" s="21" t="n">
+        <v>99.994218</v>
+      </c>
+      <c r="F1099" s="21" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="G1099" s="21" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="H1099" s="22" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="I1099" s="22" t="n">
+        <v>5999653.11</v>
+      </c>
+      <c r="J1099" s="19" t="n">
+        <v>46108</v>
+      </c>
+      <c r="K1099" s="19" t="n">
+        <v>46473</v>
+      </c>
+      <c r="L1099" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1099" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1099" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="23" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B1100" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1100" s="24" t="n">
+        <v>2464</v>
+      </c>
+      <c r="D1100" s="16" t="inlineStr">
+        <is>
+          <t>Mas de 5</t>
+        </is>
+      </c>
+      <c r="E1100" s="25" t="n">
+        <v>99.981662</v>
+      </c>
+      <c r="F1100" s="25" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="G1100" s="25" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="H1100" s="26" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="I1100" s="26" t="n">
+        <v>2999449.85</v>
+      </c>
+      <c r="J1100" s="23" t="n">
+        <v>46119</v>
+      </c>
+      <c r="K1100" s="23" t="n">
+        <v>48676</v>
+      </c>
+      <c r="L1100" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1100" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1100" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="19" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B1101" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1101" s="20" t="n">
+        <v>1017</v>
+      </c>
+      <c r="D1101" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1101" s="21" t="n">
+        <v>99.981658</v>
+      </c>
+      <c r="F1101" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1101" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1101" s="22" t="n">
+        <v>1022456</v>
+      </c>
+      <c r="I1101" s="22" t="n">
+        <v>1022268.46</v>
+      </c>
+      <c r="J1101" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1101" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1101" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1101" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1101" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="23" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1102" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1102" s="24" t="n">
+        <v>982</v>
+      </c>
+      <c r="D1102" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1102" s="25" t="n">
+        <v>99.979951</v>
+      </c>
+      <c r="F1102" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1102" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1102" s="26" t="n">
+        <v>361910</v>
+      </c>
+      <c r="I1102" s="26" t="n">
+        <v>361837.44</v>
+      </c>
+      <c r="J1102" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1102" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1102" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1102" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1102" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="19" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1103" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1103" s="20" t="n">
+        <v>982</v>
+      </c>
+      <c r="D1103" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1103" s="21" t="n">
+        <v>99.979951</v>
+      </c>
+      <c r="F1103" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1103" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1103" s="22" t="n">
+        <v>11738</v>
+      </c>
+      <c r="I1103" s="22" t="n">
+        <v>11735.65</v>
+      </c>
+      <c r="J1103" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1103" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1103" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1103" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1103" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="23" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1104" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1104" s="24" t="n">
+        <v>982</v>
+      </c>
+      <c r="D1104" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1104" s="25" t="n">
+        <v>99.979951</v>
+      </c>
+      <c r="F1104" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1104" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1104" s="26" t="n">
+        <v>110530</v>
+      </c>
+      <c r="I1104" s="26" t="n">
+        <v>110507.84</v>
+      </c>
+      <c r="J1104" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1104" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1104" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1104" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1104" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="19" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1105" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1105" s="20" t="n">
+        <v>982</v>
+      </c>
+      <c r="D1105" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1105" s="21" t="n">
+        <v>99.979951</v>
+      </c>
+      <c r="F1105" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1105" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1105" s="22" t="n">
+        <v>281200</v>
+      </c>
+      <c r="I1105" s="22" t="n">
+        <v>281143.62</v>
+      </c>
+      <c r="J1105" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1105" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1105" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1105" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1105" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="23" t="n">
+        <v>46178</v>
+      </c>
+      <c r="B1106" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1106" s="24" t="n">
+        <v>982</v>
+      </c>
+      <c r="D1106" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1106" s="25" t="n">
+        <v>99.979951</v>
+      </c>
+      <c r="F1106" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1106" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1106" s="26" t="n">
+        <v>281200</v>
+      </c>
+      <c r="I1106" s="26" t="n">
+        <v>281143.62</v>
+      </c>
+      <c r="J1106" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1106" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1106" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1106" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1106" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="19" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B1107" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1107" s="20" t="n">
+        <v>979</v>
+      </c>
+      <c r="D1107" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1107" s="21" t="n">
+        <v>99.98008900000001</v>
+      </c>
+      <c r="F1107" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1107" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1107" s="22" t="n">
+        <v>790540</v>
+      </c>
+      <c r="I1107" s="22" t="n">
+        <v>790382.6</v>
+      </c>
+      <c r="J1107" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1107" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1107" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1107" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1107" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="23" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B1108" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1108" s="24" t="n">
+        <v>978</v>
+      </c>
+      <c r="D1108" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1108" s="25" t="n">
+        <v>99.98014499999999</v>
+      </c>
+      <c r="F1108" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1108" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1108" s="26" t="n">
+        <v>60000</v>
+      </c>
+      <c r="I1108" s="26" t="n">
+        <v>59988.09</v>
+      </c>
+      <c r="J1108" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1108" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1108" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1108" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1108" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="19" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B1109" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1109" s="20" t="n">
+        <v>1012</v>
+      </c>
+      <c r="D1109" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1109" s="21" t="n">
+        <v>99.981041</v>
+      </c>
+      <c r="F1109" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1109" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1109" s="22" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="I1109" s="22" t="n">
+        <v>3999241.64</v>
+      </c>
+      <c r="J1109" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1109" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1109" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1109" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1109" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="23" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B1110" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1110" s="24" t="n">
+        <v>1011</v>
+      </c>
+      <c r="D1110" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1110" s="25" t="n">
+        <v>99.98093299999999</v>
+      </c>
+      <c r="F1110" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1110" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1110" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I1110" s="26" t="n">
+        <v>499904.66</v>
+      </c>
+      <c r="J1110" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1110" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1110" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1110" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1110" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="19" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B1111" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1111" s="20" t="n">
+        <v>977</v>
+      </c>
+      <c r="D1111" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1111" s="21" t="n">
+        <v>99.980206</v>
+      </c>
+      <c r="F1111" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1111" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1111" s="22" t="n">
+        <v>26990</v>
+      </c>
+      <c r="I1111" s="22" t="n">
+        <v>26984.66</v>
+      </c>
+      <c r="J1111" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1111" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1111" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1111" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1111" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="23" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B1112" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1112" s="24" t="n">
+        <v>977</v>
+      </c>
+      <c r="D1112" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1112" s="25" t="n">
+        <v>99.980206</v>
+      </c>
+      <c r="F1112" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1112" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1112" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1112" s="26" t="n">
+        <v>99980.21000000001</v>
+      </c>
+      <c r="J1112" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1112" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1112" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1112" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1112" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
update: deuda interna — 185 new rows, total 4.21B USD (Jun 2026)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 11-Jun-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 19-Jun-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,13 +845,13 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1751774360.969999</v>
+        <v>1761517226.16</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>536138968.9900001</v>
+        <v>543538968.99</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1170652109.64</v>
+        <v>1172994974.83</v>
       </c>
       <c r="E9" s="9" t="n">
         <v>20685165.52</v>
@@ -860,19 +860,19 @@
         <v>24298116.82</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>30.60548098746731</v>
+        <v>30.85629597701306</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>66.82664935179103</v>
+        <v>66.59003712311447</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>1.180812208516748</v>
+        <v>1.174281194234609</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.387057452224929</v>
+        <v>1.379385705637885</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.421304347826086</v>
+        <v>7.44672808219178</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4200417203.839999</v>
+        <v>4210160069.029999</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -2325,13 +2325,13 @@
         </is>
       </c>
       <c r="C57" s="9" t="n">
-        <v>27817713.82</v>
+        <v>37560579.01000001</v>
       </c>
       <c r="D57" s="9" t="n">
-        <v>15999082.69</v>
+        <v>23399082.69</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>8819181.280000001</v>
+        <v>11162046.47000001</v>
       </c>
       <c r="F57" s="9" t="n">
         <v>0</v>
@@ -3844,16 +3844,16 @@
         </is>
       </c>
       <c r="C68" s="7" t="n">
-        <v>6.75</v>
+        <v>5.4829</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>8.1073</v>
+        <v>8.1069</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>8.7117</v>
+        <v>8.667999999999999</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>9.382999999999999</v>
+        <v>9.2433</v>
       </c>
     </row>
   </sheetData>
@@ -3870,7 +3870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1112"/>
+  <dimension ref="A1:N1128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -63884,6 +63884,870 @@
         </is>
       </c>
     </row>
+    <row r="1113">
+      <c r="A1113" s="19" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B1113" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1113" s="20" t="n">
+        <v>323</v>
+      </c>
+      <c r="D1113" s="15" t="inlineStr">
+        <is>
+          <t>Hasta 1</t>
+        </is>
+      </c>
+      <c r="E1113" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1113" s="21" t="n">
+        <v>4.4853</v>
+      </c>
+      <c r="G1113" s="21" t="n">
+        <v>4.49</v>
+      </c>
+      <c r="H1113" s="22" t="n">
+        <v>7400000</v>
+      </c>
+      <c r="I1113" s="22" t="n">
+        <v>7400000</v>
+      </c>
+      <c r="J1113" s="19" t="n">
+        <v>46146</v>
+      </c>
+      <c r="K1113" s="19" t="n">
+        <v>46511</v>
+      </c>
+      <c r="L1113" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1113" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1113" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="23" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B1114" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1114" s="24" t="n">
+        <v>975</v>
+      </c>
+      <c r="D1114" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1114" s="25" t="n">
+        <v>99.99994700000001</v>
+      </c>
+      <c r="F1114" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1114" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1114" s="26" t="n">
+        <v>45000</v>
+      </c>
+      <c r="I1114" s="26" t="n">
+        <v>44999.98</v>
+      </c>
+      <c r="J1114" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1114" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1114" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1114" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1114" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="19" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B1115" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1115" s="20" t="n">
+        <v>1009</v>
+      </c>
+      <c r="D1115" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1115" s="21" t="n">
+        <v>99.99995800000001</v>
+      </c>
+      <c r="F1115" s="21" t="n">
+        <v>8.1122</v>
+      </c>
+      <c r="G1115" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1115" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1115" s="22" t="n">
+        <v>99999.96000000001</v>
+      </c>
+      <c r="J1115" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1115" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1115" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1115" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1115" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="23" t="n">
+        <v>46185</v>
+      </c>
+      <c r="B1116" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1116" s="24" t="n">
+        <v>975</v>
+      </c>
+      <c r="D1116" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1116" s="25" t="n">
+        <v>99.99994700000001</v>
+      </c>
+      <c r="F1116" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1116" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1116" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1116" s="26" t="n">
+        <v>9999.99</v>
+      </c>
+      <c r="J1116" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1116" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1116" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1116" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1116" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="19" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B1117" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1117" s="20" t="n">
+        <v>972</v>
+      </c>
+      <c r="D1117" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1117" s="21" t="n">
+        <v>99.999898</v>
+      </c>
+      <c r="F1117" s="21" t="n">
+        <v>8.1119</v>
+      </c>
+      <c r="G1117" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1117" s="22" t="n">
+        <v>271322</v>
+      </c>
+      <c r="I1117" s="22" t="n">
+        <v>271321.72</v>
+      </c>
+      <c r="J1117" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1117" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1117" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1117" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1117" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="23" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B1118" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1118" s="24" t="n">
+        <v>972</v>
+      </c>
+      <c r="D1118" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1118" s="25" t="n">
+        <v>99.999898</v>
+      </c>
+      <c r="F1118" s="25" t="n">
+        <v>8.1119</v>
+      </c>
+      <c r="G1118" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1118" s="26" t="n">
+        <v>18544</v>
+      </c>
+      <c r="I1118" s="26" t="n">
+        <v>18543.98</v>
+      </c>
+      <c r="J1118" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1118" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1118" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1118" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1118" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="19" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B1119" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1119" s="20" t="n">
+        <v>972</v>
+      </c>
+      <c r="D1119" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1119" s="21" t="n">
+        <v>99.999898</v>
+      </c>
+      <c r="F1119" s="21" t="n">
+        <v>8.1119</v>
+      </c>
+      <c r="G1119" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1119" s="22" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1119" s="22" t="n">
+        <v>19999.98</v>
+      </c>
+      <c r="J1119" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1119" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1119" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1119" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1119" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="23" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B1120" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1120" s="24" t="n">
+        <v>972</v>
+      </c>
+      <c r="D1120" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1120" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1120" s="25" t="n">
+        <v>8.1119</v>
+      </c>
+      <c r="G1120" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1120" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1120" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="J1120" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1120" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1120" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1120" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1120" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="19" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B1121" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1121" s="20" t="n">
+        <v>971</v>
+      </c>
+      <c r="D1121" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1121" s="21" t="n">
+        <v>99.999971</v>
+      </c>
+      <c r="F1121" s="21" t="n">
+        <v>8.1119</v>
+      </c>
+      <c r="G1121" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1121" s="22" t="n">
+        <v>144000</v>
+      </c>
+      <c r="I1121" s="22" t="n">
+        <v>143999.96</v>
+      </c>
+      <c r="J1121" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1121" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1121" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1121" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1121" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="23" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B1122" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1122" s="24" t="n">
+        <v>1005</v>
+      </c>
+      <c r="D1122" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1122" s="25" t="n">
+        <v>100.000038</v>
+      </c>
+      <c r="F1122" s="25" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1122" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1122" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1122" s="26" t="n">
+        <v>1000000.38</v>
+      </c>
+      <c r="J1122" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1122" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1122" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1122" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1122" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="19" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B1123" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1123" s="20" t="n">
+        <v>1004</v>
+      </c>
+      <c r="D1123" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1123" s="21" t="n">
+        <v>99.99994700000001</v>
+      </c>
+      <c r="F1123" s="21" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1123" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1123" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1123" s="22" t="n">
+        <v>14999.99</v>
+      </c>
+      <c r="J1123" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1123" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1123" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1123" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1123" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="23" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1124" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1124" s="24" t="n">
+        <v>969</v>
+      </c>
+      <c r="D1124" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1124" s="25" t="n">
+        <v>99.999894</v>
+      </c>
+      <c r="F1124" s="25" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1124" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1124" s="26" t="n">
+        <v>36000</v>
+      </c>
+      <c r="I1124" s="26" t="n">
+        <v>35999.96</v>
+      </c>
+      <c r="J1124" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1124" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1124" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1124" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1124" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="19" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1125" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1125" s="20" t="n">
+        <v>969</v>
+      </c>
+      <c r="D1125" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1125" s="21" t="n">
+        <v>99.999894</v>
+      </c>
+      <c r="F1125" s="21" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1125" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1125" s="22" t="n">
+        <v>31000</v>
+      </c>
+      <c r="I1125" s="22" t="n">
+        <v>30999.97</v>
+      </c>
+      <c r="J1125" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1125" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1125" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1125" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1125" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="23" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1126" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1126" s="24" t="n">
+        <v>969</v>
+      </c>
+      <c r="D1126" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1126" s="25" t="n">
+        <v>99.999894</v>
+      </c>
+      <c r="F1126" s="25" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1126" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1126" s="26" t="n">
+        <v>67000</v>
+      </c>
+      <c r="I1126" s="26" t="n">
+        <v>66999.92999999999</v>
+      </c>
+      <c r="J1126" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1126" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1126" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1126" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1126" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="19" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1127" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1127" s="20" t="n">
+        <v>1003</v>
+      </c>
+      <c r="D1127" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1127" s="21" t="n">
+        <v>99.999861</v>
+      </c>
+      <c r="F1127" s="21" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1127" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1127" s="22" t="n">
+        <v>135000</v>
+      </c>
+      <c r="I1127" s="22" t="n">
+        <v>134999.81</v>
+      </c>
+      <c r="J1127" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1127" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1127" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1127" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1127" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="23" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1128" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1128" s="24" t="n">
+        <v>969</v>
+      </c>
+      <c r="D1128" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1128" s="25" t="n">
+        <v>99.999894</v>
+      </c>
+      <c r="F1128" s="25" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1128" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1128" s="26" t="n">
+        <v>400000</v>
+      </c>
+      <c r="I1128" s="26" t="n">
+        <v>399999.58</v>
+      </c>
+      <c r="J1128" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1128" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1128" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1128" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1128" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
update: deuda interna — 219 new rows, total 4.22B USD (Jun 2026)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 19-Jun-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 01-Jul-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,34 +845,34 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1761517226.16</v>
+        <v>1772459705.840001</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>543538968.99</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1172994974.83</v>
+        <v>1183313461.770001</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>20685165.52</v>
+        <v>21309158.26</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>24298116.82</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>30.85629597701306</v>
+        <v>30.6658011575167</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>66.59003712311447</v>
+        <v>66.76109238879465</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>1.174281194234609</v>
+        <v>1.202236541106654</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.379385705637885</v>
+        <v>1.370869912582001</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.44672808219178</v>
+        <v>7.518256748466258</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4210160069.029999</v>
+        <v>4221102548.71</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -2325,16 +2325,16 @@
         </is>
       </c>
       <c r="C57" s="9" t="n">
-        <v>37560579.01000001</v>
+        <v>48503058.69000001</v>
       </c>
       <c r="D57" s="9" t="n">
         <v>23399082.69</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>11162046.47000001</v>
+        <v>21480533.41000001</v>
       </c>
       <c r="F57" s="9" t="n">
-        <v>0</v>
+        <v>623992.74</v>
       </c>
       <c r="G57" s="9" t="n">
         <v>2999449.85</v>
@@ -3844,16 +3844,16 @@
         </is>
       </c>
       <c r="C68" s="7" t="n">
-        <v>5.4829</v>
+        <v>5.663</v>
       </c>
       <c r="D68" s="7" t="n">
-        <v>8.1069</v>
+        <v>8.0832</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>8.667999999999999</v>
+        <v>8.628299999999999</v>
       </c>
       <c r="F68" s="7" t="n">
-        <v>9.2433</v>
+        <v>9.1974</v>
       </c>
     </row>
   </sheetData>
@@ -3870,7 +3870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1128"/>
+  <dimension ref="A1:N1162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64748,6 +64748,1842 @@
         </is>
       </c>
     </row>
+    <row r="1129">
+      <c r="A1129" s="19" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B1129" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1129" s="20" t="n">
+        <v>968</v>
+      </c>
+      <c r="D1129" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1129" s="21" t="n">
+        <v>99.999982</v>
+      </c>
+      <c r="F1129" s="21" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1129" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1129" s="22" t="n">
+        <v>35000</v>
+      </c>
+      <c r="I1129" s="22" t="n">
+        <v>34999.99</v>
+      </c>
+      <c r="J1129" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1129" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1129" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1129" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1129" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="23" t="n">
+        <v>46192</v>
+      </c>
+      <c r="B1130" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1130" s="24" t="n">
+        <v>968</v>
+      </c>
+      <c r="D1130" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1130" s="25" t="n">
+        <v>99.999982</v>
+      </c>
+      <c r="F1130" s="25" t="n">
+        <v>8.112</v>
+      </c>
+      <c r="G1130" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1130" s="26" t="n">
+        <v>39000</v>
+      </c>
+      <c r="I1130" s="26" t="n">
+        <v>38999.99</v>
+      </c>
+      <c r="J1130" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1130" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1130" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1130" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1130" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="19" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B1131" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1131" s="20" t="n">
+        <v>965</v>
+      </c>
+      <c r="D1131" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1131" s="21" t="n">
+        <v>99.999803</v>
+      </c>
+      <c r="F1131" s="21" t="n">
+        <v>8.1122</v>
+      </c>
+      <c r="G1131" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1131" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1131" s="22" t="n">
+        <v>14999.97</v>
+      </c>
+      <c r="J1131" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1131" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1131" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1131" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1131" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="23" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B1132" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1132" s="24" t="n">
+        <v>965</v>
+      </c>
+      <c r="D1132" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1132" s="25" t="n">
+        <v>99.999803</v>
+      </c>
+      <c r="F1132" s="25" t="n">
+        <v>8.1122</v>
+      </c>
+      <c r="G1132" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1132" s="26" t="n">
+        <v>63000</v>
+      </c>
+      <c r="I1132" s="26" t="n">
+        <v>62999.88</v>
+      </c>
+      <c r="J1132" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1132" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1132" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1132" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1132" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="19" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B1133" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1133" s="20" t="n">
+        <v>965</v>
+      </c>
+      <c r="D1133" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1133" s="21" t="n">
+        <v>99.999803</v>
+      </c>
+      <c r="F1133" s="21" t="n">
+        <v>8.1122</v>
+      </c>
+      <c r="G1133" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1133" s="22" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1133" s="22" t="n">
+        <v>49999.9</v>
+      </c>
+      <c r="J1133" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1133" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1133" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1133" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1133" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="23" t="n">
+        <v>46195</v>
+      </c>
+      <c r="B1134" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1134" s="24" t="n">
+        <v>999</v>
+      </c>
+      <c r="D1134" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1134" s="25" t="n">
+        <v>99.99981</v>
+      </c>
+      <c r="F1134" s="25" t="n">
+        <v>8.1119</v>
+      </c>
+      <c r="G1134" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1134" s="26" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I1134" s="26" t="n">
+        <v>39999.92</v>
+      </c>
+      <c r="J1134" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1134" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1134" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1134" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1134" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="19" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1135" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1135" s="20" t="n">
+        <v>963</v>
+      </c>
+      <c r="D1135" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1135" s="21" t="n">
+        <v>99.99978900000001</v>
+      </c>
+      <c r="F1135" s="21" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1135" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1135" s="22" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="I1135" s="22" t="n">
+        <v>2999993.68</v>
+      </c>
+      <c r="J1135" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1135" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1135" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1135" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1135" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="23" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1136" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1136" s="24" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1136" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1136" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1136" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1136" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1136" s="26" t="n">
+        <v>750000</v>
+      </c>
+      <c r="I1136" s="26" t="n">
+        <v>750000</v>
+      </c>
+      <c r="J1136" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1136" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1136" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1136" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1136" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="19" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1137" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1137" s="20" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1137" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1137" s="21" t="n">
+        <v>99.99993600000001</v>
+      </c>
+      <c r="F1137" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1137" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1137" s="22" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1137" s="22" t="n">
+        <v>49999.97</v>
+      </c>
+      <c r="J1137" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1137" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1137" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1137" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1137" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="23" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1138" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1138" s="24" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D1138" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1138" s="25" t="n">
+        <v>99.99968200000001</v>
+      </c>
+      <c r="F1138" s="25" t="n">
+        <v>8.2852</v>
+      </c>
+      <c r="G1138" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1138" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1138" s="26" t="n">
+        <v>99999.67999999999</v>
+      </c>
+      <c r="J1138" s="23" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1138" s="23" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1138" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1138" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1138" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="19" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1139" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1139" s="20" t="n">
+        <v>1679</v>
+      </c>
+      <c r="D1139" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1139" s="21" t="n">
+        <v>99.99968200000001</v>
+      </c>
+      <c r="F1139" s="21" t="n">
+        <v>8.2852</v>
+      </c>
+      <c r="G1139" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1139" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1139" s="22" t="n">
+        <v>99999.67999999999</v>
+      </c>
+      <c r="J1139" s="19" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1139" s="19" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1139" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1139" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1139" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="23" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1140" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1140" s="24" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1140" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1140" s="25" t="n">
+        <v>99.99993600000001</v>
+      </c>
+      <c r="F1140" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1140" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1140" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1140" s="26" t="n">
+        <v>29999.98</v>
+      </c>
+      <c r="J1140" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1140" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1140" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1140" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1140" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="19" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1141" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1141" s="20" t="n">
+        <v>997</v>
+      </c>
+      <c r="D1141" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1141" s="21" t="n">
+        <v>99.99993600000001</v>
+      </c>
+      <c r="F1141" s="21" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1141" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1141" s="22" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1141" s="22" t="n">
+        <v>29999.98</v>
+      </c>
+      <c r="J1141" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1141" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1141" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1141" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1141" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="23" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1142" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1142" s="24" t="n">
+        <v>962</v>
+      </c>
+      <c r="D1142" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1142" s="25" t="n">
+        <v>99.999908</v>
+      </c>
+      <c r="F1142" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1142" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1142" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1142" s="26" t="n">
+        <v>49999.95</v>
+      </c>
+      <c r="J1142" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1142" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1142" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1142" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1142" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="19" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1143" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1143" s="20" t="n">
+        <v>962</v>
+      </c>
+      <c r="D1143" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1143" s="21" t="n">
+        <v>99.999908</v>
+      </c>
+      <c r="F1143" s="21" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1143" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1143" s="22" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I1143" s="22" t="n">
+        <v>24999.98</v>
+      </c>
+      <c r="J1143" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1143" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1143" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1143" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1143" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="23" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1144" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1144" s="24" t="n">
+        <v>962</v>
+      </c>
+      <c r="D1144" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1144" s="25" t="n">
+        <v>99.999908</v>
+      </c>
+      <c r="F1144" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1144" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1144" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1144" s="26" t="n">
+        <v>29999.97</v>
+      </c>
+      <c r="J1144" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1144" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1144" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1144" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1144" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="19" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1145" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1145" s="20" t="n">
+        <v>962</v>
+      </c>
+      <c r="D1145" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1145" s="21" t="n">
+        <v>99.999908</v>
+      </c>
+      <c r="F1145" s="21" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1145" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1145" s="22" t="n">
+        <v>56000</v>
+      </c>
+      <c r="I1145" s="22" t="n">
+        <v>55999.95</v>
+      </c>
+      <c r="J1145" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1145" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1145" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1145" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1145" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="23" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1146" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1146" s="24" t="n">
+        <v>962</v>
+      </c>
+      <c r="D1146" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1146" s="25" t="n">
+        <v>99.999908</v>
+      </c>
+      <c r="F1146" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1146" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1146" s="26" t="n">
+        <v>194000</v>
+      </c>
+      <c r="I1146" s="26" t="n">
+        <v>193999.82</v>
+      </c>
+      <c r="J1146" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1146" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1146" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1146" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1146" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="19" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1147" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1147" s="20" t="n">
+        <v>962</v>
+      </c>
+      <c r="D1147" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1147" s="21" t="n">
+        <v>99.999908</v>
+      </c>
+      <c r="F1147" s="21" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1147" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1147" s="22" t="n">
+        <v>29000</v>
+      </c>
+      <c r="I1147" s="22" t="n">
+        <v>28999.97</v>
+      </c>
+      <c r="J1147" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1147" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1147" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1147" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1147" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="23" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1148" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1148" s="24" t="n">
+        <v>1678</v>
+      </c>
+      <c r="D1148" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1148" s="25" t="n">
+        <v>99.999836</v>
+      </c>
+      <c r="F1148" s="25" t="n">
+        <v>8.2852</v>
+      </c>
+      <c r="G1148" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1148" s="26" t="n">
+        <v>193000</v>
+      </c>
+      <c r="I1148" s="26" t="n">
+        <v>192999.68</v>
+      </c>
+      <c r="J1148" s="23" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1148" s="23" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1148" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1148" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1148" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="19" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1149" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1149" s="20" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1149" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1149" s="21" t="n">
+        <v>99.999796</v>
+      </c>
+      <c r="F1149" s="21" t="n">
+        <v>8.112399999999999</v>
+      </c>
+      <c r="G1149" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1149" s="22" t="n">
+        <v>29000</v>
+      </c>
+      <c r="I1149" s="22" t="n">
+        <v>28999.94</v>
+      </c>
+      <c r="J1149" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1149" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1149" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1149" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1149" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="23" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1150" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1150" s="24" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1150" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1150" s="25" t="n">
+        <v>99.999796</v>
+      </c>
+      <c r="F1150" s="25" t="n">
+        <v>8.112399999999999</v>
+      </c>
+      <c r="G1150" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1150" s="26" t="n">
+        <v>27000</v>
+      </c>
+      <c r="I1150" s="26" t="n">
+        <v>26999.95</v>
+      </c>
+      <c r="J1150" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1150" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1150" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1150" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1150" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="19" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1151" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1151" s="20" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1151" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1151" s="21" t="n">
+        <v>99.999796</v>
+      </c>
+      <c r="F1151" s="21" t="n">
+        <v>8.112399999999999</v>
+      </c>
+      <c r="G1151" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1151" s="22" t="n">
+        <v>113000</v>
+      </c>
+      <c r="I1151" s="22" t="n">
+        <v>112999.77</v>
+      </c>
+      <c r="J1151" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1151" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1151" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1151" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1151" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="23" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1152" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1152" s="24" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1152" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1152" s="25" t="n">
+        <v>100.000032</v>
+      </c>
+      <c r="F1152" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1152" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1152" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1152" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="J1152" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1152" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1152" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1152" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1152" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="19" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1153" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1153" s="20" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1153" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1153" s="21" t="n">
+        <v>100.000032</v>
+      </c>
+      <c r="F1153" s="21" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1153" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1153" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1153" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J1153" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1153" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1153" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1153" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1153" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="23" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1154" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1154" s="24" t="n">
+        <v>995</v>
+      </c>
+      <c r="D1154" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1154" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1154" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1154" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1154" s="26" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I1154" s="26" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J1154" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1154" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1154" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1154" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1154" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="19" t="n">
+        <v>46199</v>
+      </c>
+      <c r="B1155" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1155" s="20" t="n">
+        <v>1677</v>
+      </c>
+      <c r="D1155" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1155" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1155" s="21" t="n">
+        <v>8.2852</v>
+      </c>
+      <c r="G1155" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1155" s="22" t="n">
+        <v>230993.7</v>
+      </c>
+      <c r="I1155" s="22" t="n">
+        <v>230993.7</v>
+      </c>
+      <c r="J1155" s="19" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1155" s="19" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1155" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1155" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1155" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="23" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B1156" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1156" s="24" t="n">
+        <v>958</v>
+      </c>
+      <c r="D1156" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1156" s="25" t="n">
+        <v>99.99996400000001</v>
+      </c>
+      <c r="F1156" s="25" t="n">
+        <v>8.112500000000001</v>
+      </c>
+      <c r="G1156" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1156" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1156" s="26" t="n">
+        <v>99999.96000000001</v>
+      </c>
+      <c r="J1156" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1156" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1156" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1156" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1156" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="19" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B1157" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1157" s="20" t="n">
+        <v>992</v>
+      </c>
+      <c r="D1157" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1157" s="21" t="n">
+        <v>99.99997</v>
+      </c>
+      <c r="F1157" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1157" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1157" s="22" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I1157" s="22" t="n">
+        <v>199999.94</v>
+      </c>
+      <c r="J1157" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1157" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1157" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1157" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1157" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="23" t="n">
+        <v>46202</v>
+      </c>
+      <c r="B1158" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1158" s="24" t="n">
+        <v>958</v>
+      </c>
+      <c r="D1158" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1158" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1158" s="25" t="n">
+        <v>8.112500000000001</v>
+      </c>
+      <c r="G1158" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1158" s="26" t="n">
+        <v>184500</v>
+      </c>
+      <c r="I1158" s="26" t="n">
+        <v>184500</v>
+      </c>
+      <c r="J1158" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1158" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1158" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1158" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1158" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="19" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B1159" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1159" s="20" t="n">
+        <v>957</v>
+      </c>
+      <c r="D1159" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1159" s="21" t="n">
+        <v>99.99987299999999</v>
+      </c>
+      <c r="F1159" s="21" t="n">
+        <v>8.1126</v>
+      </c>
+      <c r="G1159" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1159" s="22" t="n">
+        <v>1343000</v>
+      </c>
+      <c r="I1159" s="22" t="n">
+        <v>1342998.3</v>
+      </c>
+      <c r="J1159" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1159" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1159" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1159" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1159" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="23" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B1160" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1160" s="24" t="n">
+        <v>957</v>
+      </c>
+      <c r="D1160" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1160" s="25" t="n">
+        <v>99.99987299999999</v>
+      </c>
+      <c r="F1160" s="25" t="n">
+        <v>8.1126</v>
+      </c>
+      <c r="G1160" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1160" s="26" t="n">
+        <v>2411000</v>
+      </c>
+      <c r="I1160" s="26" t="n">
+        <v>2410996.94</v>
+      </c>
+      <c r="J1160" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1160" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1160" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1160" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1160" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="19" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B1161" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1161" s="20" t="n">
+        <v>957</v>
+      </c>
+      <c r="D1161" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1161" s="21" t="n">
+        <v>99.99987299999999</v>
+      </c>
+      <c r="F1161" s="21" t="n">
+        <v>8.1126</v>
+      </c>
+      <c r="G1161" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1161" s="22" t="n">
+        <v>600000</v>
+      </c>
+      <c r="I1161" s="22" t="n">
+        <v>599999.24</v>
+      </c>
+      <c r="J1161" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1161" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1161" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1161" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1161" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="23" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B1162" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1162" s="24" t="n">
+        <v>957</v>
+      </c>
+      <c r="D1162" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1162" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1162" s="25" t="n">
+        <v>8.112500000000001</v>
+      </c>
+      <c r="G1162" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1162" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I1162" s="26" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1162" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1162" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1162" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1162" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1162" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
update: deuda interna — 1525 new rows, total 4.32B USD (Jul 2026)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 01-Jul-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 03-Aug-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,34 +845,34 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1772459705.840001</v>
+        <v>1872646092.690002</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>543538968.99</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1183313461.770001</v>
+        <v>1259151251.600002</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>21309158.26</v>
+        <v>45519118.66</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>24298116.82</v>
+        <v>24436753.44</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>30.6658011575167</v>
+        <v>29.02518372861485</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>66.76109238879465</v>
+        <v>67.23914660197579</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>1.202236541106654</v>
+        <v>2.430737918803072</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.370869912582001</v>
+        <v>1.304931750606294</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.518256748466258</v>
+        <v>7.597657978723404</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4221102548.71</v>
+        <v>4321288935.560001</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -909,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2325,19 +2325,44 @@
         </is>
       </c>
       <c r="C57" s="9" t="n">
-        <v>48503058.69000001</v>
+        <v>49503058.69000001</v>
       </c>
       <c r="D57" s="9" t="n">
         <v>23399082.69</v>
       </c>
       <c r="E57" s="9" t="n">
-        <v>21480533.41000001</v>
+        <v>22480533.41000001</v>
       </c>
       <c r="F57" s="9" t="n">
         <v>623992.74</v>
       </c>
       <c r="G57" s="9" t="n">
         <v>2999449.85</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="n">
+        <v>99186386.84999996</v>
+      </c>
+      <c r="D58" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="5" t="n">
+        <v>74837789.82999997</v>
+      </c>
+      <c r="F58" s="5" t="n">
+        <v>24209960.4</v>
+      </c>
+      <c r="G58" s="5" t="n">
+        <v>138636.62</v>
       </c>
     </row>
   </sheetData>
@@ -2354,7 +2379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3850,10 +3875,54 @@
         <v>8.0832</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>8.628299999999999</v>
+        <v>8.6309</v>
       </c>
       <c r="F68" s="7" t="n">
         <v>9.1974</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B69" s="15" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="C69" s="11" t="n">
+        <v>5.8916</v>
+      </c>
+      <c r="D69" s="11" t="n">
+        <v>7.5972</v>
+      </c>
+      <c r="E69" s="11" t="n">
+        <v>8.7163</v>
+      </c>
+      <c r="F69" s="11" t="n">
+        <v>9.183999999999999</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>Ago</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="D70" s="7" t="n">
+        <v>6.6235</v>
+      </c>
+      <c r="E70" s="7" t="n">
+        <v>8.535</v>
+      </c>
+      <c r="F70" s="7" t="n">
+        <v>9.375</v>
       </c>
     </row>
   </sheetData>
@@ -3870,7 +3939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1162"/>
+  <dimension ref="A1:N1212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -64426,7 +64495,7 @@
     </row>
     <row r="1123">
       <c r="A1123" s="19" t="n">
-        <v>46190</v>
+        <v>46189</v>
       </c>
       <c r="B1123" s="15" t="inlineStr">
         <is>
@@ -64434,7 +64503,7 @@
         </is>
       </c>
       <c r="C1123" s="20" t="n">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="D1123" s="15" t="inlineStr">
         <is>
@@ -64442,7 +64511,7 @@
         </is>
       </c>
       <c r="E1123" s="21" t="n">
-        <v>99.99994700000001</v>
+        <v>100</v>
       </c>
       <c r="F1123" s="21" t="n">
         <v>8.112</v>
@@ -64451,10 +64520,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1123" s="22" t="n">
-        <v>15000</v>
+        <v>1000000</v>
       </c>
       <c r="I1123" s="22" t="n">
-        <v>14999.99</v>
+        <v>1000000</v>
       </c>
       <c r="J1123" s="19" t="n">
         <v>46113</v>
@@ -64480,7 +64549,7 @@
     </row>
     <row r="1124">
       <c r="A1124" s="23" t="n">
-        <v>46191</v>
+        <v>46190</v>
       </c>
       <c r="B1124" s="16" t="inlineStr">
         <is>
@@ -64488,7 +64557,7 @@
         </is>
       </c>
       <c r="C1124" s="24" t="n">
-        <v>969</v>
+        <v>1004</v>
       </c>
       <c r="D1124" s="16" t="inlineStr">
         <is>
@@ -64496,7 +64565,7 @@
         </is>
       </c>
       <c r="E1124" s="25" t="n">
-        <v>99.999894</v>
+        <v>99.99994700000001</v>
       </c>
       <c r="F1124" s="25" t="n">
         <v>8.112</v>
@@ -64505,16 +64574,16 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1124" s="26" t="n">
-        <v>36000</v>
+        <v>15000</v>
       </c>
       <c r="I1124" s="26" t="n">
-        <v>35999.96</v>
+        <v>14999.99</v>
       </c>
       <c r="J1124" s="23" t="n">
-        <v>46080</v>
+        <v>46113</v>
       </c>
       <c r="K1124" s="23" t="n">
-        <v>47176</v>
+        <v>47209</v>
       </c>
       <c r="L1124" s="16" t="inlineStr">
         <is>
@@ -64559,10 +64628,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1125" s="22" t="n">
-        <v>31000</v>
+        <v>36000</v>
       </c>
       <c r="I1125" s="22" t="n">
-        <v>30999.97</v>
+        <v>35999.96</v>
       </c>
       <c r="J1125" s="19" t="n">
         <v>46080</v>
@@ -64613,10 +64682,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1126" s="26" t="n">
-        <v>67000</v>
+        <v>31000</v>
       </c>
       <c r="I1126" s="26" t="n">
-        <v>66999.92999999999</v>
+        <v>30999.97</v>
       </c>
       <c r="J1126" s="23" t="n">
         <v>46080</v>
@@ -64650,7 +64719,7 @@
         </is>
       </c>
       <c r="C1127" s="20" t="n">
-        <v>1003</v>
+        <v>969</v>
       </c>
       <c r="D1127" s="15" t="inlineStr">
         <is>
@@ -64658,7 +64727,7 @@
         </is>
       </c>
       <c r="E1127" s="21" t="n">
-        <v>99.999861</v>
+        <v>99.999894</v>
       </c>
       <c r="F1127" s="21" t="n">
         <v>8.112</v>
@@ -64667,16 +64736,16 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1127" s="22" t="n">
-        <v>135000</v>
+        <v>67000</v>
       </c>
       <c r="I1127" s="22" t="n">
-        <v>134999.81</v>
+        <v>66999.92999999999</v>
       </c>
       <c r="J1127" s="19" t="n">
-        <v>46113</v>
+        <v>46080</v>
       </c>
       <c r="K1127" s="19" t="n">
-        <v>47209</v>
+        <v>47176</v>
       </c>
       <c r="L1127" s="15" t="inlineStr">
         <is>
@@ -64704,7 +64773,7 @@
         </is>
       </c>
       <c r="C1128" s="24" t="n">
-        <v>969</v>
+        <v>1003</v>
       </c>
       <c r="D1128" s="16" t="inlineStr">
         <is>
@@ -64712,7 +64781,7 @@
         </is>
       </c>
       <c r="E1128" s="25" t="n">
-        <v>99.999894</v>
+        <v>99.999861</v>
       </c>
       <c r="F1128" s="25" t="n">
         <v>8.112</v>
@@ -64721,16 +64790,16 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1128" s="26" t="n">
-        <v>400000</v>
+        <v>135000</v>
       </c>
       <c r="I1128" s="26" t="n">
-        <v>399999.58</v>
+        <v>134999.81</v>
       </c>
       <c r="J1128" s="23" t="n">
-        <v>46080</v>
+        <v>46113</v>
       </c>
       <c r="K1128" s="23" t="n">
-        <v>47176</v>
+        <v>47209</v>
       </c>
       <c r="L1128" s="16" t="inlineStr">
         <is>
@@ -64750,7 +64819,7 @@
     </row>
     <row r="1129">
       <c r="A1129" s="19" t="n">
-        <v>46192</v>
+        <v>46191</v>
       </c>
       <c r="B1129" s="15" t="inlineStr">
         <is>
@@ -64758,7 +64827,7 @@
         </is>
       </c>
       <c r="C1129" s="20" t="n">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="D1129" s="15" t="inlineStr">
         <is>
@@ -64766,7 +64835,7 @@
         </is>
       </c>
       <c r="E1129" s="21" t="n">
-        <v>99.999982</v>
+        <v>99.999894</v>
       </c>
       <c r="F1129" s="21" t="n">
         <v>8.112</v>
@@ -64775,10 +64844,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1129" s="22" t="n">
-        <v>35000</v>
+        <v>400000</v>
       </c>
       <c r="I1129" s="22" t="n">
-        <v>34999.99</v>
+        <v>399999.58</v>
       </c>
       <c r="J1129" s="19" t="n">
         <v>46080</v>
@@ -64829,10 +64898,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1130" s="26" t="n">
-        <v>39000</v>
+        <v>35000</v>
       </c>
       <c r="I1130" s="26" t="n">
-        <v>38999.99</v>
+        <v>34999.99</v>
       </c>
       <c r="J1130" s="23" t="n">
         <v>46080</v>
@@ -64842,7 +64911,7 @@
       </c>
       <c r="L1130" s="16" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1130" s="16" t="inlineStr">
@@ -64858,7 +64927,7 @@
     </row>
     <row r="1131">
       <c r="A1131" s="19" t="n">
-        <v>46195</v>
+        <v>46192</v>
       </c>
       <c r="B1131" s="15" t="inlineStr">
         <is>
@@ -64866,7 +64935,7 @@
         </is>
       </c>
       <c r="C1131" s="20" t="n">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="D1131" s="15" t="inlineStr">
         <is>
@@ -64874,19 +64943,19 @@
         </is>
       </c>
       <c r="E1131" s="21" t="n">
-        <v>99.999803</v>
+        <v>99.999982</v>
       </c>
       <c r="F1131" s="21" t="n">
-        <v>8.1122</v>
+        <v>8.112</v>
       </c>
       <c r="G1131" s="21" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1131" s="22" t="n">
-        <v>15000</v>
+        <v>39000</v>
       </c>
       <c r="I1131" s="22" t="n">
-        <v>14999.97</v>
+        <v>38999.99</v>
       </c>
       <c r="J1131" s="19" t="n">
         <v>46080</v>
@@ -64896,7 +64965,7 @@
       </c>
       <c r="L1131" s="15" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M1131" s="15" t="inlineStr">
@@ -64937,10 +65006,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1132" s="26" t="n">
-        <v>63000</v>
+        <v>15000</v>
       </c>
       <c r="I1132" s="26" t="n">
-        <v>62999.88</v>
+        <v>14999.97</v>
       </c>
       <c r="J1132" s="23" t="n">
         <v>46080</v>
@@ -64991,10 +65060,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1133" s="22" t="n">
-        <v>50000</v>
+        <v>63000</v>
       </c>
       <c r="I1133" s="22" t="n">
-        <v>49999.9</v>
+        <v>62999.88</v>
       </c>
       <c r="J1133" s="19" t="n">
         <v>46080</v>
@@ -65004,7 +65073,7 @@
       </c>
       <c r="L1133" s="15" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1133" s="15" t="inlineStr">
@@ -65028,7 +65097,7 @@
         </is>
       </c>
       <c r="C1134" s="24" t="n">
-        <v>999</v>
+        <v>965</v>
       </c>
       <c r="D1134" s="16" t="inlineStr">
         <is>
@@ -65036,29 +65105,29 @@
         </is>
       </c>
       <c r="E1134" s="25" t="n">
-        <v>99.99981</v>
+        <v>99.999803</v>
       </c>
       <c r="F1134" s="25" t="n">
-        <v>8.1119</v>
+        <v>8.1122</v>
       </c>
       <c r="G1134" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1134" s="26" t="n">
-        <v>40000</v>
+        <v>50000</v>
       </c>
       <c r="I1134" s="26" t="n">
-        <v>39999.92</v>
+        <v>49999.9</v>
       </c>
       <c r="J1134" s="23" t="n">
-        <v>46113</v>
+        <v>46080</v>
       </c>
       <c r="K1134" s="23" t="n">
-        <v>47209</v>
+        <v>47176</v>
       </c>
       <c r="L1134" s="16" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M1134" s="16" t="inlineStr">
@@ -65074,7 +65143,7 @@
     </row>
     <row r="1135">
       <c r="A1135" s="19" t="n">
-        <v>46197</v>
+        <v>46195</v>
       </c>
       <c r="B1135" s="15" t="inlineStr">
         <is>
@@ -65082,7 +65151,7 @@
         </is>
       </c>
       <c r="C1135" s="20" t="n">
-        <v>963</v>
+        <v>999</v>
       </c>
       <c r="D1135" s="15" t="inlineStr">
         <is>
@@ -65090,25 +65159,25 @@
         </is>
       </c>
       <c r="E1135" s="21" t="n">
-        <v>99.99978900000001</v>
+        <v>99.99981</v>
       </c>
       <c r="F1135" s="21" t="n">
-        <v>8.112299999999999</v>
+        <v>8.1119</v>
       </c>
       <c r="G1135" s="21" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1135" s="22" t="n">
-        <v>3000000</v>
+        <v>40000</v>
       </c>
       <c r="I1135" s="22" t="n">
-        <v>2999993.68</v>
+        <v>39999.92</v>
       </c>
       <c r="J1135" s="19" t="n">
-        <v>46080</v>
+        <v>46113</v>
       </c>
       <c r="K1135" s="19" t="n">
-        <v>47176</v>
+        <v>47209</v>
       </c>
       <c r="L1135" s="15" t="inlineStr">
         <is>
@@ -65136,7 +65205,7 @@
         </is>
       </c>
       <c r="C1136" s="24" t="n">
-        <v>997</v>
+        <v>963</v>
       </c>
       <c r="D1136" s="16" t="inlineStr">
         <is>
@@ -65144,29 +65213,29 @@
         </is>
       </c>
       <c r="E1136" s="25" t="n">
-        <v>100</v>
+        <v>99.99978900000001</v>
       </c>
       <c r="F1136" s="25" t="n">
-        <v>8.111800000000001</v>
+        <v>8.112299999999999</v>
       </c>
       <c r="G1136" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1136" s="26" t="n">
-        <v>750000</v>
+        <v>3000000</v>
       </c>
       <c r="I1136" s="26" t="n">
-        <v>750000</v>
+        <v>2999993.68</v>
       </c>
       <c r="J1136" s="23" t="n">
-        <v>46113</v>
+        <v>46080</v>
       </c>
       <c r="K1136" s="23" t="n">
-        <v>47209</v>
+        <v>47176</v>
       </c>
       <c r="L1136" s="16" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1136" s="16" t="inlineStr">
@@ -65198,7 +65267,7 @@
         </is>
       </c>
       <c r="E1137" s="21" t="n">
-        <v>99.99993600000001</v>
+        <v>100</v>
       </c>
       <c r="F1137" s="21" t="n">
         <v>8.111800000000001</v>
@@ -65207,10 +65276,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1137" s="22" t="n">
-        <v>50000</v>
+        <v>750000</v>
       </c>
       <c r="I1137" s="22" t="n">
-        <v>49999.97</v>
+        <v>750000</v>
       </c>
       <c r="J1137" s="19" t="n">
         <v>46113</v>
@@ -65220,7 +65289,7 @@
       </c>
       <c r="L1137" s="15" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M1137" s="15" t="inlineStr">
@@ -65244,33 +65313,33 @@
         </is>
       </c>
       <c r="C1138" s="24" t="n">
-        <v>1679</v>
+        <v>997</v>
       </c>
       <c r="D1138" s="16" t="inlineStr">
         <is>
-          <t>De 3 a 5</t>
+          <t>De 1 a 3</t>
         </is>
       </c>
       <c r="E1138" s="25" t="n">
-        <v>99.99968200000001</v>
+        <v>99.99993600000001</v>
       </c>
       <c r="F1138" s="25" t="n">
-        <v>8.2852</v>
+        <v>8.111800000000001</v>
       </c>
       <c r="G1138" s="25" t="n">
-        <v>8.289999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="H1138" s="26" t="n">
-        <v>100000</v>
+        <v>50000</v>
       </c>
       <c r="I1138" s="26" t="n">
-        <v>99999.67999999999</v>
+        <v>49999.97</v>
       </c>
       <c r="J1138" s="23" t="n">
-        <v>46076</v>
+        <v>46113</v>
       </c>
       <c r="K1138" s="23" t="n">
-        <v>47902</v>
+        <v>47209</v>
       </c>
       <c r="L1138" s="16" t="inlineStr">
         <is>
@@ -65352,33 +65421,33 @@
         </is>
       </c>
       <c r="C1140" s="24" t="n">
-        <v>997</v>
+        <v>1679</v>
       </c>
       <c r="D1140" s="16" t="inlineStr">
         <is>
-          <t>De 1 a 3</t>
+          <t>De 3 a 5</t>
         </is>
       </c>
       <c r="E1140" s="25" t="n">
-        <v>99.99993600000001</v>
+        <v>99.99968200000001</v>
       </c>
       <c r="F1140" s="25" t="n">
-        <v>8.111800000000001</v>
+        <v>8.2852</v>
       </c>
       <c r="G1140" s="25" t="n">
-        <v>8.119999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="H1140" s="26" t="n">
-        <v>30000</v>
+        <v>100000</v>
       </c>
       <c r="I1140" s="26" t="n">
-        <v>29999.98</v>
+        <v>99999.67999999999</v>
       </c>
       <c r="J1140" s="23" t="n">
-        <v>46113</v>
+        <v>46076</v>
       </c>
       <c r="K1140" s="23" t="n">
-        <v>47209</v>
+        <v>47902</v>
       </c>
       <c r="L1140" s="16" t="inlineStr">
         <is>
@@ -65452,7 +65521,7 @@
     </row>
     <row r="1142">
       <c r="A1142" s="23" t="n">
-        <v>46198</v>
+        <v>46197</v>
       </c>
       <c r="B1142" s="16" t="inlineStr">
         <is>
@@ -65460,7 +65529,7 @@
         </is>
       </c>
       <c r="C1142" s="24" t="n">
-        <v>962</v>
+        <v>997</v>
       </c>
       <c r="D1142" s="16" t="inlineStr">
         <is>
@@ -65468,29 +65537,29 @@
         </is>
       </c>
       <c r="E1142" s="25" t="n">
-        <v>99.999908</v>
+        <v>99.99993600000001</v>
       </c>
       <c r="F1142" s="25" t="n">
-        <v>8.112299999999999</v>
+        <v>8.111800000000001</v>
       </c>
       <c r="G1142" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1142" s="26" t="n">
-        <v>50000</v>
+        <v>30000</v>
       </c>
       <c r="I1142" s="26" t="n">
-        <v>49999.95</v>
+        <v>29999.98</v>
       </c>
       <c r="J1142" s="23" t="n">
-        <v>46080</v>
+        <v>46113</v>
       </c>
       <c r="K1142" s="23" t="n">
-        <v>47176</v>
+        <v>47209</v>
       </c>
       <c r="L1142" s="16" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1142" s="16" t="inlineStr">
@@ -65531,10 +65600,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1143" s="22" t="n">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="I1143" s="22" t="n">
-        <v>24999.98</v>
+        <v>49999.95</v>
       </c>
       <c r="J1143" s="19" t="n">
         <v>46080</v>
@@ -65585,10 +65654,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1144" s="26" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="I1144" s="26" t="n">
-        <v>29999.97</v>
+        <v>24999.98</v>
       </c>
       <c r="J1144" s="23" t="n">
         <v>46080</v>
@@ -65598,7 +65667,7 @@
       </c>
       <c r="L1144" s="16" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M1144" s="16" t="inlineStr">
@@ -65639,10 +65708,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1145" s="22" t="n">
-        <v>56000</v>
+        <v>30000</v>
       </c>
       <c r="I1145" s="22" t="n">
-        <v>55999.95</v>
+        <v>29999.97</v>
       </c>
       <c r="J1145" s="19" t="n">
         <v>46080</v>
@@ -65693,10 +65762,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1146" s="26" t="n">
-        <v>194000</v>
+        <v>56000</v>
       </c>
       <c r="I1146" s="26" t="n">
-        <v>193999.82</v>
+        <v>55999.95</v>
       </c>
       <c r="J1146" s="23" t="n">
         <v>46080</v>
@@ -65747,10 +65816,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1147" s="22" t="n">
-        <v>29000</v>
+        <v>194000</v>
       </c>
       <c r="I1147" s="22" t="n">
-        <v>28999.97</v>
+        <v>193999.82</v>
       </c>
       <c r="J1147" s="19" t="n">
         <v>46080</v>
@@ -65784,33 +65853,33 @@
         </is>
       </c>
       <c r="C1148" s="24" t="n">
-        <v>1678</v>
+        <v>962</v>
       </c>
       <c r="D1148" s="16" t="inlineStr">
         <is>
-          <t>De 3 a 5</t>
+          <t>De 1 a 3</t>
         </is>
       </c>
       <c r="E1148" s="25" t="n">
-        <v>99.999836</v>
+        <v>99.999908</v>
       </c>
       <c r="F1148" s="25" t="n">
-        <v>8.2852</v>
+        <v>8.112299999999999</v>
       </c>
       <c r="G1148" s="25" t="n">
-        <v>8.289999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="H1148" s="26" t="n">
-        <v>193000</v>
+        <v>29000</v>
       </c>
       <c r="I1148" s="26" t="n">
-        <v>192999.68</v>
+        <v>28999.97</v>
       </c>
       <c r="J1148" s="23" t="n">
-        <v>46076</v>
+        <v>46080</v>
       </c>
       <c r="K1148" s="23" t="n">
-        <v>47902</v>
+        <v>47176</v>
       </c>
       <c r="L1148" s="16" t="inlineStr">
         <is>
@@ -65830,7 +65899,7 @@
     </row>
     <row r="1149">
       <c r="A1149" s="19" t="n">
-        <v>46199</v>
+        <v>46198</v>
       </c>
       <c r="B1149" s="15" t="inlineStr">
         <is>
@@ -65838,33 +65907,33 @@
         </is>
       </c>
       <c r="C1149" s="20" t="n">
-        <v>961</v>
+        <v>1678</v>
       </c>
       <c r="D1149" s="15" t="inlineStr">
         <is>
-          <t>De 1 a 3</t>
+          <t>De 3 a 5</t>
         </is>
       </c>
       <c r="E1149" s="21" t="n">
-        <v>99.999796</v>
+        <v>99.999836</v>
       </c>
       <c r="F1149" s="21" t="n">
-        <v>8.112399999999999</v>
+        <v>8.2852</v>
       </c>
       <c r="G1149" s="21" t="n">
-        <v>8.119999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="H1149" s="22" t="n">
-        <v>29000</v>
+        <v>193000</v>
       </c>
       <c r="I1149" s="22" t="n">
-        <v>28999.94</v>
+        <v>192999.68</v>
       </c>
       <c r="J1149" s="19" t="n">
-        <v>46080</v>
+        <v>46076</v>
       </c>
       <c r="K1149" s="19" t="n">
-        <v>47176</v>
+        <v>47902</v>
       </c>
       <c r="L1149" s="15" t="inlineStr">
         <is>
@@ -65909,10 +65978,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1150" s="26" t="n">
-        <v>27000</v>
+        <v>29000</v>
       </c>
       <c r="I1150" s="26" t="n">
-        <v>26999.95</v>
+        <v>28999.94</v>
       </c>
       <c r="J1150" s="23" t="n">
         <v>46080</v>
@@ -65963,10 +66032,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1151" s="22" t="n">
-        <v>113000</v>
+        <v>27000</v>
       </c>
       <c r="I1151" s="22" t="n">
-        <v>112999.77</v>
+        <v>26999.95</v>
       </c>
       <c r="J1151" s="19" t="n">
         <v>46080</v>
@@ -66008,19 +66077,19 @@
         </is>
       </c>
       <c r="E1152" s="25" t="n">
-        <v>100.000032</v>
+        <v>99.999796</v>
       </c>
       <c r="F1152" s="25" t="n">
-        <v>8.112299999999999</v>
+        <v>8.112399999999999</v>
       </c>
       <c r="G1152" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1152" s="26" t="n">
-        <v>15000</v>
+        <v>113000</v>
       </c>
       <c r="I1152" s="26" t="n">
-        <v>15000</v>
+        <v>112999.77</v>
       </c>
       <c r="J1152" s="23" t="n">
         <v>46080</v>
@@ -66030,7 +66099,7 @@
       </c>
       <c r="L1152" s="16" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1152" s="16" t="inlineStr">
@@ -66071,10 +66140,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1153" s="22" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="I1153" s="22" t="n">
-        <v>10000</v>
+        <v>15000</v>
       </c>
       <c r="J1153" s="19" t="n">
         <v>46080</v>
@@ -66108,7 +66177,7 @@
         </is>
       </c>
       <c r="C1154" s="24" t="n">
-        <v>995</v>
+        <v>961</v>
       </c>
       <c r="D1154" s="16" t="inlineStr">
         <is>
@@ -66116,25 +66185,25 @@
         </is>
       </c>
       <c r="E1154" s="25" t="n">
-        <v>100</v>
+        <v>100.000032</v>
       </c>
       <c r="F1154" s="25" t="n">
-        <v>8.111700000000001</v>
+        <v>8.112299999999999</v>
       </c>
       <c r="G1154" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1154" s="26" t="n">
-        <v>300000</v>
+        <v>10000</v>
       </c>
       <c r="I1154" s="26" t="n">
-        <v>300000</v>
+        <v>10000</v>
       </c>
       <c r="J1154" s="23" t="n">
-        <v>46113</v>
+        <v>46080</v>
       </c>
       <c r="K1154" s="23" t="n">
-        <v>47209</v>
+        <v>47176</v>
       </c>
       <c r="L1154" s="16" t="inlineStr">
         <is>
@@ -66162,33 +66231,33 @@
         </is>
       </c>
       <c r="C1155" s="20" t="n">
-        <v>1677</v>
+        <v>995</v>
       </c>
       <c r="D1155" s="15" t="inlineStr">
         <is>
-          <t>De 3 a 5</t>
+          <t>De 1 a 3</t>
         </is>
       </c>
       <c r="E1155" s="21" t="n">
         <v>100</v>
       </c>
       <c r="F1155" s="21" t="n">
-        <v>8.2852</v>
+        <v>8.111700000000001</v>
       </c>
       <c r="G1155" s="21" t="n">
-        <v>8.289999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="H1155" s="22" t="n">
-        <v>230993.7</v>
+        <v>300000</v>
       </c>
       <c r="I1155" s="22" t="n">
-        <v>230993.7</v>
+        <v>300000</v>
       </c>
       <c r="J1155" s="19" t="n">
-        <v>46076</v>
+        <v>46113</v>
       </c>
       <c r="K1155" s="19" t="n">
-        <v>47902</v>
+        <v>47209</v>
       </c>
       <c r="L1155" s="15" t="inlineStr">
         <is>
@@ -66208,7 +66277,7 @@
     </row>
     <row r="1156">
       <c r="A1156" s="23" t="n">
-        <v>46202</v>
+        <v>46199</v>
       </c>
       <c r="B1156" s="16" t="inlineStr">
         <is>
@@ -66216,37 +66285,37 @@
         </is>
       </c>
       <c r="C1156" s="24" t="n">
-        <v>958</v>
+        <v>1677</v>
       </c>
       <c r="D1156" s="16" t="inlineStr">
         <is>
-          <t>De 1 a 3</t>
+          <t>De 3 a 5</t>
         </is>
       </c>
       <c r="E1156" s="25" t="n">
-        <v>99.99996400000001</v>
+        <v>100</v>
       </c>
       <c r="F1156" s="25" t="n">
-        <v>8.112500000000001</v>
+        <v>8.2852</v>
       </c>
       <c r="G1156" s="25" t="n">
-        <v>8.119999999999999</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="H1156" s="26" t="n">
-        <v>100000</v>
+        <v>230993.7</v>
       </c>
       <c r="I1156" s="26" t="n">
-        <v>99999.96000000001</v>
+        <v>230993.7</v>
       </c>
       <c r="J1156" s="23" t="n">
-        <v>46080</v>
+        <v>46076</v>
       </c>
       <c r="K1156" s="23" t="n">
-        <v>47176</v>
+        <v>47902</v>
       </c>
       <c r="L1156" s="16" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M1156" s="16" t="inlineStr">
@@ -66270,7 +66339,7 @@
         </is>
       </c>
       <c r="C1157" s="20" t="n">
-        <v>992</v>
+        <v>958</v>
       </c>
       <c r="D1157" s="15" t="inlineStr">
         <is>
@@ -66278,25 +66347,25 @@
         </is>
       </c>
       <c r="E1157" s="21" t="n">
-        <v>99.99997</v>
+        <v>99.99996400000001</v>
       </c>
       <c r="F1157" s="21" t="n">
-        <v>8.111700000000001</v>
+        <v>8.112500000000001</v>
       </c>
       <c r="G1157" s="21" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1157" s="22" t="n">
-        <v>200000</v>
+        <v>100000</v>
       </c>
       <c r="I1157" s="22" t="n">
-        <v>199999.94</v>
+        <v>99999.96000000001</v>
       </c>
       <c r="J1157" s="19" t="n">
-        <v>46113</v>
+        <v>46080</v>
       </c>
       <c r="K1157" s="19" t="n">
-        <v>47209</v>
+        <v>47176</v>
       </c>
       <c r="L1157" s="15" t="inlineStr">
         <is>
@@ -66324,7 +66393,7 @@
         </is>
       </c>
       <c r="C1158" s="24" t="n">
-        <v>958</v>
+        <v>992</v>
       </c>
       <c r="D1158" s="16" t="inlineStr">
         <is>
@@ -66332,29 +66401,29 @@
         </is>
       </c>
       <c r="E1158" s="25" t="n">
-        <v>100</v>
+        <v>99.99997</v>
       </c>
       <c r="F1158" s="25" t="n">
-        <v>8.112500000000001</v>
+        <v>8.111700000000001</v>
       </c>
       <c r="G1158" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1158" s="26" t="n">
-        <v>184500</v>
+        <v>200000</v>
       </c>
       <c r="I1158" s="26" t="n">
-        <v>184500</v>
+        <v>199999.94</v>
       </c>
       <c r="J1158" s="23" t="n">
-        <v>46080</v>
+        <v>46113</v>
       </c>
       <c r="K1158" s="23" t="n">
-        <v>47176</v>
+        <v>47209</v>
       </c>
       <c r="L1158" s="16" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1158" s="16" t="inlineStr">
@@ -66370,7 +66439,7 @@
     </row>
     <row r="1159">
       <c r="A1159" s="19" t="n">
-        <v>46203</v>
+        <v>46202</v>
       </c>
       <c r="B1159" s="15" t="inlineStr">
         <is>
@@ -66378,7 +66447,7 @@
         </is>
       </c>
       <c r="C1159" s="20" t="n">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="D1159" s="15" t="inlineStr">
         <is>
@@ -66386,19 +66455,19 @@
         </is>
       </c>
       <c r="E1159" s="21" t="n">
-        <v>99.99987299999999</v>
+        <v>100</v>
       </c>
       <c r="F1159" s="21" t="n">
-        <v>8.1126</v>
+        <v>8.112500000000001</v>
       </c>
       <c r="G1159" s="21" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1159" s="22" t="n">
-        <v>1343000</v>
+        <v>184500</v>
       </c>
       <c r="I1159" s="22" t="n">
-        <v>1342998.3</v>
+        <v>184500</v>
       </c>
       <c r="J1159" s="19" t="n">
         <v>46080</v>
@@ -66408,7 +66477,7 @@
       </c>
       <c r="L1159" s="15" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>Q</t>
         </is>
       </c>
       <c r="M1159" s="15" t="inlineStr">
@@ -66449,10 +66518,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1160" s="26" t="n">
-        <v>2411000</v>
+        <v>1343000</v>
       </c>
       <c r="I1160" s="26" t="n">
-        <v>2410996.94</v>
+        <v>1342998.3</v>
       </c>
       <c r="J1160" s="23" t="n">
         <v>46080</v>
@@ -66462,7 +66531,7 @@
       </c>
       <c r="L1160" s="16" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M1160" s="16" t="inlineStr">
@@ -66503,10 +66572,10 @@
         <v>8.119999999999999</v>
       </c>
       <c r="H1161" s="22" t="n">
-        <v>600000</v>
+        <v>2411000</v>
       </c>
       <c r="I1161" s="22" t="n">
-        <v>599999.24</v>
+        <v>2410996.94</v>
       </c>
       <c r="J1161" s="19" t="n">
         <v>46080</v>
@@ -66548,19 +66617,19 @@
         </is>
       </c>
       <c r="E1162" s="25" t="n">
-        <v>100</v>
+        <v>99.99987299999999</v>
       </c>
       <c r="F1162" s="25" t="n">
-        <v>8.112500000000001</v>
+        <v>8.1126</v>
       </c>
       <c r="G1162" s="25" t="n">
         <v>8.119999999999999</v>
       </c>
       <c r="H1162" s="26" t="n">
-        <v>500000</v>
+        <v>600000</v>
       </c>
       <c r="I1162" s="26" t="n">
-        <v>500000</v>
+        <v>599999.24</v>
       </c>
       <c r="J1162" s="23" t="n">
         <v>46080</v>
@@ -66579,6 +66648,2706 @@
         </is>
       </c>
       <c r="N1162" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="19" t="n">
+        <v>46203</v>
+      </c>
+      <c r="B1163" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1163" s="20" t="n">
+        <v>957</v>
+      </c>
+      <c r="D1163" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1163" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1163" s="21" t="n">
+        <v>8.112500000000001</v>
+      </c>
+      <c r="G1163" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1163" s="22" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I1163" s="22" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J1163" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1163" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1163" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1163" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1163" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="23" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1164" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1164" s="24" t="n">
+        <v>956</v>
+      </c>
+      <c r="D1164" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1164" s="25" t="n">
+        <v>100.000023</v>
+      </c>
+      <c r="F1164" s="25" t="n">
+        <v>8.1126</v>
+      </c>
+      <c r="G1164" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1164" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1164" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J1164" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1164" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1164" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1164" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1164" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="19" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1165" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1165" s="20" t="n">
+        <v>956</v>
+      </c>
+      <c r="D1165" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1165" s="21" t="n">
+        <v>99.999788</v>
+      </c>
+      <c r="F1165" s="21" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1165" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1165" s="22" t="n">
+        <v>43665</v>
+      </c>
+      <c r="I1165" s="22" t="n">
+        <v>43664.91</v>
+      </c>
+      <c r="J1165" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1165" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1165" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1165" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1165" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="23" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1166" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1166" s="24" t="n">
+        <v>956</v>
+      </c>
+      <c r="D1166" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1166" s="25" t="n">
+        <v>99.999788</v>
+      </c>
+      <c r="F1166" s="25" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1166" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1166" s="26" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1166" s="26" t="n">
+        <v>99999.78999999999</v>
+      </c>
+      <c r="J1166" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1166" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1166" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1166" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1166" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" s="19" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1167" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1167" s="20" t="n">
+        <v>956</v>
+      </c>
+      <c r="D1167" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1167" s="21" t="n">
+        <v>99.999788</v>
+      </c>
+      <c r="F1167" s="21" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1167" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1167" s="22" t="n">
+        <v>45000</v>
+      </c>
+      <c r="I1167" s="22" t="n">
+        <v>44999.9</v>
+      </c>
+      <c r="J1167" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1167" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1167" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1167" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1167" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="23" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1168" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1168" s="24" t="n">
+        <v>956</v>
+      </c>
+      <c r="D1168" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1168" s="25" t="n">
+        <v>99.999788</v>
+      </c>
+      <c r="F1168" s="25" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1168" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1168" s="26" t="n">
+        <v>27000</v>
+      </c>
+      <c r="I1168" s="26" t="n">
+        <v>26999.94</v>
+      </c>
+      <c r="J1168" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1168" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1168" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1168" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1168" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="19" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1169" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1169" s="20" t="n">
+        <v>956</v>
+      </c>
+      <c r="D1169" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1169" s="21" t="n">
+        <v>99.999788</v>
+      </c>
+      <c r="F1169" s="21" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1169" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1169" s="22" t="n">
+        <v>23000</v>
+      </c>
+      <c r="I1169" s="22" t="n">
+        <v>22999.95</v>
+      </c>
+      <c r="J1169" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1169" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1169" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1169" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1169" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="23" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B1170" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1170" s="24" t="n">
+        <v>955</v>
+      </c>
+      <c r="D1170" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1170" s="25" t="n">
+        <v>99.999943</v>
+      </c>
+      <c r="F1170" s="25" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1170" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1170" s="26" t="n">
+        <v>98000</v>
+      </c>
+      <c r="I1170" s="26" t="n">
+        <v>97999.94</v>
+      </c>
+      <c r="J1170" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1170" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1170" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1170" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1170" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="19" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B1171" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1171" s="20" t="n">
+        <v>955</v>
+      </c>
+      <c r="D1171" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1171" s="21" t="n">
+        <v>99.999943</v>
+      </c>
+      <c r="F1171" s="21" t="n">
+        <v>8.1127</v>
+      </c>
+      <c r="G1171" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1171" s="22" t="n">
+        <v>59000</v>
+      </c>
+      <c r="I1171" s="22" t="n">
+        <v>58999.97</v>
+      </c>
+      <c r="J1171" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1171" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1171" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1171" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1171" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="23" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B1172" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1172" s="24" t="n">
+        <v>980</v>
+      </c>
+      <c r="D1172" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1172" s="25" t="n">
+        <v>99.999973</v>
+      </c>
+      <c r="F1172" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1172" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1172" s="26" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="I1172" s="26" t="n">
+        <v>1999999.47</v>
+      </c>
+      <c r="J1172" s="23" t="n">
+        <v>46104</v>
+      </c>
+      <c r="K1172" s="23" t="n">
+        <v>47200</v>
+      </c>
+      <c r="L1172" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1172" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1172" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="19" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B1173" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1173" s="20" t="n">
+        <v>980</v>
+      </c>
+      <c r="D1173" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1173" s="21" t="n">
+        <v>99.999973</v>
+      </c>
+      <c r="F1173" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1173" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1173" s="22" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="I1173" s="22" t="n">
+        <v>7999997.86</v>
+      </c>
+      <c r="J1173" s="19" t="n">
+        <v>46104</v>
+      </c>
+      <c r="K1173" s="19" t="n">
+        <v>47200</v>
+      </c>
+      <c r="L1173" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1173" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1173" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="23" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B1174" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1174" s="24" t="n">
+        <v>954</v>
+      </c>
+      <c r="D1174" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1174" s="25" t="n">
+        <v>99.99986800000001</v>
+      </c>
+      <c r="F1174" s="25" t="n">
+        <v>8.1128</v>
+      </c>
+      <c r="G1174" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1174" s="26" t="n">
+        <v>14000</v>
+      </c>
+      <c r="I1174" s="26" t="n">
+        <v>13999.98</v>
+      </c>
+      <c r="J1174" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1174" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1174" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1174" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1174" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="19" t="n">
+        <v>46206</v>
+      </c>
+      <c r="B1175" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1175" s="20" t="n">
+        <v>980</v>
+      </c>
+      <c r="D1175" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1175" s="21" t="n">
+        <v>99.999973</v>
+      </c>
+      <c r="F1175" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1175" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1175" s="22" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="I1175" s="22" t="n">
+        <v>19999994.65</v>
+      </c>
+      <c r="J1175" s="19" t="n">
+        <v>46104</v>
+      </c>
+      <c r="K1175" s="19" t="n">
+        <v>47200</v>
+      </c>
+      <c r="L1175" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1175" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1175" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="23" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B1176" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1176" s="24" t="n">
+        <v>984</v>
+      </c>
+      <c r="D1176" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1176" s="25" t="n">
+        <v>99.999892</v>
+      </c>
+      <c r="F1176" s="25" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1176" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1176" s="26" t="n">
+        <v>250000</v>
+      </c>
+      <c r="I1176" s="26" t="n">
+        <v>249999.73</v>
+      </c>
+      <c r="J1176" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1176" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1176" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1176" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1176" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="19" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B1177" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1177" s="20" t="n">
+        <v>984</v>
+      </c>
+      <c r="D1177" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1177" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1177" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1177" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1177" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I1177" s="22" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J1177" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1177" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1177" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1177" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1177" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="23" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B1178" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1178" s="24" t="n">
+        <v>948</v>
+      </c>
+      <c r="D1178" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1178" s="25" t="n">
+        <v>100.000003</v>
+      </c>
+      <c r="F1178" s="25" t="n">
+        <v>8.113200000000001</v>
+      </c>
+      <c r="G1178" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1178" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1178" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J1178" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1178" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1178" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1178" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1178" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="19" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B1179" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1179" s="20" t="n">
+        <v>948</v>
+      </c>
+      <c r="D1179" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1179" s="21" t="n">
+        <v>99.99977</v>
+      </c>
+      <c r="F1179" s="21" t="n">
+        <v>8.113300000000001</v>
+      </c>
+      <c r="G1179" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1179" s="22" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="I1179" s="22" t="n">
+        <v>9999976.960000001</v>
+      </c>
+      <c r="J1179" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1179" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1179" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1179" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1179" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="23" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B1180" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1180" s="24" t="n">
+        <v>978</v>
+      </c>
+      <c r="D1180" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1180" s="25" t="n">
+        <v>99.999804</v>
+      </c>
+      <c r="F1180" s="25" t="n">
+        <v>8.111800000000001</v>
+      </c>
+      <c r="G1180" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1180" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1180" s="26" t="n">
+        <v>19999.96</v>
+      </c>
+      <c r="J1180" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1180" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1180" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1180" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1180" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="19" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B1181" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1181" s="20" t="n">
+        <v>977</v>
+      </c>
+      <c r="D1181" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1181" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1181" s="21" t="n">
+        <v>8.111700000000001</v>
+      </c>
+      <c r="G1181" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1181" s="22" t="n">
+        <v>150000</v>
+      </c>
+      <c r="I1181" s="22" t="n">
+        <v>150000</v>
+      </c>
+      <c r="J1181" s="19" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1181" s="19" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1181" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1181" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1181" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="23" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B1182" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1182" s="24" t="n">
+        <v>943</v>
+      </c>
+      <c r="D1182" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1182" s="25" t="n">
+        <v>99.99987400000001</v>
+      </c>
+      <c r="F1182" s="25" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1182" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1182" s="26" t="n">
+        <v>11000</v>
+      </c>
+      <c r="I1182" s="26" t="n">
+        <v>10999.99</v>
+      </c>
+      <c r="J1182" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1182" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1182" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1182" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1182" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" s="19" t="n">
+        <v>46217</v>
+      </c>
+      <c r="B1183" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1183" s="20" t="n">
+        <v>943</v>
+      </c>
+      <c r="D1183" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1183" s="21" t="n">
+        <v>99.99987400000001</v>
+      </c>
+      <c r="F1183" s="21" t="n">
+        <v>8.1137</v>
+      </c>
+      <c r="G1183" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1183" s="22" t="n">
+        <v>35000</v>
+      </c>
+      <c r="I1183" s="22" t="n">
+        <v>34999.96</v>
+      </c>
+      <c r="J1183" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1183" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1183" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1183" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1183" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" s="23" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B1184" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1184" s="24" t="n">
+        <v>2452</v>
+      </c>
+      <c r="D1184" s="16" t="inlineStr">
+        <is>
+          <t>Mas de 5</t>
+        </is>
+      </c>
+      <c r="E1184" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1184" s="25" t="n">
+        <v>8.366099999999999</v>
+      </c>
+      <c r="G1184" s="25" t="n">
+        <v>8.369999999999999</v>
+      </c>
+      <c r="H1184" s="26" t="n">
+        <v>138636.62</v>
+      </c>
+      <c r="I1184" s="26" t="n">
+        <v>138636.62</v>
+      </c>
+      <c r="J1184" s="23" t="n">
+        <v>46149</v>
+      </c>
+      <c r="K1184" s="23" t="n">
+        <v>48706</v>
+      </c>
+      <c r="L1184" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1184" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1184" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" s="19" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B1185" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1185" s="20" t="n">
+        <v>940</v>
+      </c>
+      <c r="D1185" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1185" s="21" t="n">
+        <v>99.999863</v>
+      </c>
+      <c r="F1185" s="21" t="n">
+        <v>8.114000000000001</v>
+      </c>
+      <c r="G1185" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1185" s="22" t="n">
+        <v>60000</v>
+      </c>
+      <c r="I1185" s="22" t="n">
+        <v>59999.92</v>
+      </c>
+      <c r="J1185" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1185" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1185" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1185" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1185" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" s="23" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B1186" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1186" s="24" t="n">
+        <v>937</v>
+      </c>
+      <c r="D1186" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1186" s="25" t="n">
+        <v>99.99990099999999</v>
+      </c>
+      <c r="F1186" s="25" t="n">
+        <v>8.1143</v>
+      </c>
+      <c r="G1186" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1186" s="26" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I1186" s="26" t="n">
+        <v>299999.7</v>
+      </c>
+      <c r="J1186" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1186" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1186" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1186" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1186" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" s="19" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B1187" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1187" s="20" t="n">
+        <v>937</v>
+      </c>
+      <c r="D1187" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1187" s="21" t="n">
+        <v>99.99990099999999</v>
+      </c>
+      <c r="F1187" s="21" t="n">
+        <v>8.1143</v>
+      </c>
+      <c r="G1187" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1187" s="22" t="n">
+        <v>34000</v>
+      </c>
+      <c r="I1187" s="22" t="n">
+        <v>33999.97</v>
+      </c>
+      <c r="J1187" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1187" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1187" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1187" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1187" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" s="23" t="n">
+        <v>46223</v>
+      </c>
+      <c r="B1188" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1188" s="24" t="n">
+        <v>937</v>
+      </c>
+      <c r="D1188" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1188" s="25" t="n">
+        <v>99.99990099999999</v>
+      </c>
+      <c r="F1188" s="25" t="n">
+        <v>8.1143</v>
+      </c>
+      <c r="G1188" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1188" s="26" t="n">
+        <v>32000</v>
+      </c>
+      <c r="I1188" s="26" t="n">
+        <v>31999.97</v>
+      </c>
+      <c r="J1188" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1188" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1188" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1188" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1188" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" s="19" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B1189" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1189" s="20" t="n">
+        <v>936</v>
+      </c>
+      <c r="D1189" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1189" s="21" t="n">
+        <v>99.999925</v>
+      </c>
+      <c r="F1189" s="21" t="n">
+        <v>8.1144</v>
+      </c>
+      <c r="G1189" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1189" s="22" t="n">
+        <v>42000</v>
+      </c>
+      <c r="I1189" s="22" t="n">
+        <v>41999.97</v>
+      </c>
+      <c r="J1189" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1189" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1189" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1189" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1189" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" s="23" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B1190" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1190" s="24" t="n">
+        <v>935</v>
+      </c>
+      <c r="D1190" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1190" s="25" t="n">
+        <v>99.999954</v>
+      </c>
+      <c r="F1190" s="25" t="n">
+        <v>8.1145</v>
+      </c>
+      <c r="G1190" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1190" s="26" t="n">
+        <v>193200</v>
+      </c>
+      <c r="I1190" s="26" t="n">
+        <v>193199.91</v>
+      </c>
+      <c r="J1190" s="23" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1190" s="23" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1190" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1190" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1190" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" s="19" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B1191" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1191" s="20" t="n">
+        <v>935</v>
+      </c>
+      <c r="D1191" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1191" s="21" t="n">
+        <v>99.999954</v>
+      </c>
+      <c r="F1191" s="21" t="n">
+        <v>8.1145</v>
+      </c>
+      <c r="G1191" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1191" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1191" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J1191" s="19" t="n">
+        <v>46080</v>
+      </c>
+      <c r="K1191" s="19" t="n">
+        <v>47176</v>
+      </c>
+      <c r="L1191" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1191" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1191" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" s="23" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B1192" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1192" s="24" t="n">
+        <v>1651</v>
+      </c>
+      <c r="D1192" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1192" s="25" t="n">
+        <v>99.99995800000001</v>
+      </c>
+      <c r="F1192" s="25" t="n">
+        <v>8.286799999999999</v>
+      </c>
+      <c r="G1192" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1192" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1192" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J1192" s="23" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1192" s="23" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1192" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1192" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1192" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B1193" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1193" s="20" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D1193" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1193" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1193" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1193" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1193" s="22" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="I1193" s="22" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="J1193" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1193" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1193" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1193" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1193" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B1194" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1194" s="24" t="n">
+        <v>1080</v>
+      </c>
+      <c r="D1194" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1194" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1194" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="G1194" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1194" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1194" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J1194" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1194" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1194" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1194" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1194" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" s="19" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B1195" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1195" s="20" t="n">
+        <v>1079</v>
+      </c>
+      <c r="D1195" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1195" s="21" t="n">
+        <v>99.999818</v>
+      </c>
+      <c r="F1195" s="21" t="n">
+        <v>8.119899999999999</v>
+      </c>
+      <c r="G1195" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1195" s="22" t="n">
+        <v>59825</v>
+      </c>
+      <c r="I1195" s="22" t="n">
+        <v>59824.89</v>
+      </c>
+      <c r="J1195" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1195" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1195" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1195" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1195" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" s="23" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B1196" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1196" s="24" t="n">
+        <v>720</v>
+      </c>
+      <c r="D1196" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1196" s="25" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1196" s="25" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="G1196" s="25" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="H1196" s="26" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="I1196" s="26" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="J1196" s="23" t="n">
+        <v>46230</v>
+      </c>
+      <c r="K1196" s="23" t="n">
+        <v>46961</v>
+      </c>
+      <c r="L1196" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1196" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1196" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" s="19" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B1197" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1197" s="20" t="n">
+        <v>1079</v>
+      </c>
+      <c r="D1197" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1197" s="21" t="n">
+        <v>99.999818</v>
+      </c>
+      <c r="F1197" s="21" t="n">
+        <v>8.119899999999999</v>
+      </c>
+      <c r="G1197" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1197" s="22" t="n">
+        <v>13000000</v>
+      </c>
+      <c r="I1197" s="22" t="n">
+        <v>12999976.34</v>
+      </c>
+      <c r="J1197" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1197" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1197" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1197" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1197" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" s="23" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B1198" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1198" s="24" t="n">
+        <v>1649</v>
+      </c>
+      <c r="D1198" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1198" s="25" t="n">
+        <v>99.99982</v>
+      </c>
+      <c r="F1198" s="25" t="n">
+        <v>8.287000000000001</v>
+      </c>
+      <c r="G1198" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1198" s="26" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="I1198" s="26" t="n">
+        <v>11999978.4</v>
+      </c>
+      <c r="J1198" s="23" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1198" s="23" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1198" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1198" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1198" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" s="19" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B1199" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1199" s="20" t="n">
+        <v>1079</v>
+      </c>
+      <c r="D1199" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1199" s="21" t="n">
+        <v>100.000079</v>
+      </c>
+      <c r="F1199" s="21" t="n">
+        <v>8.1198</v>
+      </c>
+      <c r="G1199" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1199" s="22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I1199" s="22" t="n">
+        <v>3000</v>
+      </c>
+      <c r="J1199" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1199" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1199" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1199" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1199" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" s="23" t="n">
+        <v>46227</v>
+      </c>
+      <c r="B1200" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1200" s="24" t="n">
+        <v>1649</v>
+      </c>
+      <c r="D1200" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1200" s="25" t="n">
+        <v>99.99982</v>
+      </c>
+      <c r="F1200" s="25" t="n">
+        <v>8.287000000000001</v>
+      </c>
+      <c r="G1200" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1200" s="26" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="I1200" s="26" t="n">
+        <v>9999982</v>
+      </c>
+      <c r="J1200" s="23" t="n">
+        <v>46076</v>
+      </c>
+      <c r="K1200" s="23" t="n">
+        <v>47902</v>
+      </c>
+      <c r="L1200" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1200" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1200" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" s="19" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B1201" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1201" s="20" t="n">
+        <v>1076</v>
+      </c>
+      <c r="D1201" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1201" s="21" t="n">
+        <v>99.99982</v>
+      </c>
+      <c r="F1201" s="21" t="n">
+        <v>8.119400000000001</v>
+      </c>
+      <c r="G1201" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1201" s="22" t="n">
+        <v>16000</v>
+      </c>
+      <c r="I1201" s="22" t="n">
+        <v>15999.97</v>
+      </c>
+      <c r="J1201" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1201" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1201" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1201" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1201" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" s="23" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B1202" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1202" s="24" t="n">
+        <v>1075</v>
+      </c>
+      <c r="D1202" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1202" s="25" t="n">
+        <v>100.000177</v>
+      </c>
+      <c r="F1202" s="25" t="n">
+        <v>8.1191</v>
+      </c>
+      <c r="G1202" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1202" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="I1202" s="26" t="n">
+        <v>9000.02</v>
+      </c>
+      <c r="J1202" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1202" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1202" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1202" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1202" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" s="19" t="n">
+        <v>46231</v>
+      </c>
+      <c r="B1203" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1203" s="20" t="n">
+        <v>1075</v>
+      </c>
+      <c r="D1203" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1203" s="21" t="n">
+        <v>100.000177</v>
+      </c>
+      <c r="F1203" s="21" t="n">
+        <v>8.1191</v>
+      </c>
+      <c r="G1203" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1203" s="22" t="n">
+        <v>16000</v>
+      </c>
+      <c r="I1203" s="22" t="n">
+        <v>16000.03</v>
+      </c>
+      <c r="J1203" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1203" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1203" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1203" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1203" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B1204" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1204" s="24" t="n">
+        <v>1074</v>
+      </c>
+      <c r="D1204" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1204" s="25" t="n">
+        <v>100.000016</v>
+      </c>
+      <c r="F1204" s="25" t="n">
+        <v>8.119</v>
+      </c>
+      <c r="G1204" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1204" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1204" s="26" t="n">
+        <v>1000000.16</v>
+      </c>
+      <c r="J1204" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1204" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1204" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1204" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1204" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B1205" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1205" s="20" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D1205" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1205" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="F1205" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="G1205" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1205" s="22" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="I1205" s="22" t="n">
+        <v>2200000</v>
+      </c>
+      <c r="J1205" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1205" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1205" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1205" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1205" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" s="23" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B1206" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1206" s="24" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1206" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1206" s="25" t="n">
+        <v>100.000032</v>
+      </c>
+      <c r="F1206" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1206" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1206" s="26" t="n">
+        <v>845000</v>
+      </c>
+      <c r="I1206" s="26" t="n">
+        <v>845000.27</v>
+      </c>
+      <c r="J1206" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1206" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1206" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1206" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1206" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" s="19" t="n">
+        <v>46233</v>
+      </c>
+      <c r="B1207" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1207" s="20" t="n">
+        <v>1073</v>
+      </c>
+      <c r="D1207" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1207" s="21" t="n">
+        <v>100.00012</v>
+      </c>
+      <c r="F1207" s="21" t="n">
+        <v>8.1188</v>
+      </c>
+      <c r="G1207" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1207" s="22" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1207" s="22" t="n">
+        <v>1000001.2</v>
+      </c>
+      <c r="J1207" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1207" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1207" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1207" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1207" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" s="23" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B1208" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1208" s="24" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1208" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1208" s="25" t="n">
+        <v>100.000032</v>
+      </c>
+      <c r="F1208" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1208" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1208" s="26" t="n">
+        <v>491000</v>
+      </c>
+      <c r="I1208" s="26" t="n">
+        <v>491000.16</v>
+      </c>
+      <c r="J1208" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1208" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1208" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1208" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1208" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" s="19" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B1209" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1209" s="20" t="n">
+        <v>1073</v>
+      </c>
+      <c r="D1209" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1209" s="21" t="n">
+        <v>100.00012</v>
+      </c>
+      <c r="F1209" s="21" t="n">
+        <v>8.1188</v>
+      </c>
+      <c r="G1209" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1209" s="22" t="n">
+        <v>294600</v>
+      </c>
+      <c r="I1209" s="22" t="n">
+        <v>294600.35</v>
+      </c>
+      <c r="J1209" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1209" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1209" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1209" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1209" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" s="23" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B1210" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1210" s="24" t="n">
+        <v>961</v>
+      </c>
+      <c r="D1210" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1210" s="25" t="n">
+        <v>100.000032</v>
+      </c>
+      <c r="F1210" s="25" t="n">
+        <v>8.112299999999999</v>
+      </c>
+      <c r="G1210" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1210" s="26" t="n">
+        <v>90000</v>
+      </c>
+      <c r="I1210" s="26" t="n">
+        <v>90000.03</v>
+      </c>
+      <c r="J1210" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1210" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1210" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1210" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1210" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="19" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B1211" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1211" s="20" t="n">
+        <v>1073</v>
+      </c>
+      <c r="D1211" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1211" s="21" t="n">
+        <v>100.00012</v>
+      </c>
+      <c r="F1211" s="21" t="n">
+        <v>8.1188</v>
+      </c>
+      <c r="G1211" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1211" s="22" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="I1211" s="22" t="n">
+        <v>2600003.13</v>
+      </c>
+      <c r="J1211" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1211" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1211" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1211" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1211" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="23" t="n">
+        <v>46234</v>
+      </c>
+      <c r="B1212" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1212" s="24" t="n">
+        <v>1073</v>
+      </c>
+      <c r="D1212" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1212" s="25" t="n">
+        <v>100.00012</v>
+      </c>
+      <c r="F1212" s="25" t="n">
+        <v>8.1188</v>
+      </c>
+      <c r="G1212" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1212" s="26" t="n">
+        <v>726550</v>
+      </c>
+      <c r="I1212" s="26" t="n">
+        <v>726550.88</v>
+      </c>
+      <c r="J1212" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1212" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1212" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1212" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1212" s="16" t="inlineStr">
         <is>
           <t>SC</t>
         </is>

</xml_diff>

<commit_message>
update: deuda interna — 471 new rows, total 4.38B USD (Aug 2026)
</commit_message>
<xml_diff>
--- a/deuda-interna/deuda_interna_resumen.xlsx
+++ b/deuda-interna/deuda_interna_resumen.xlsx
@@ -604,7 +604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generado: 03-Aug-2026  ·  Fuente: Bolsa de Valores de Quito</t>
+          <t>Generado: 22-Aug-2026  ·  Fuente: Bolsa de Valores de Quito</t>
         </is>
       </c>
     </row>
@@ -845,34 +845,34 @@
         <v>2026</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1872646092.690002</v>
+        <v>1930761460.400001</v>
       </c>
       <c r="C9" s="9" t="n">
         <v>543538968.99</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>1259151251.600002</v>
+        <v>1314172597.270001</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>45519118.66</v>
+        <v>48613140.7</v>
       </c>
       <c r="F9" s="9" t="n">
         <v>24436753.44</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>29.02518372861485</v>
+        <v>28.15153400034169</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>67.23914660197579</v>
+        <v>68.06499012041293</v>
       </c>
       <c r="I9" s="10" t="n">
-        <v>2.430737918803072</v>
+        <v>2.51782220108789</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>1.304931750606294</v>
+        <v>1.265653678157496</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>7.597657978723404</v>
+        <v>7.672456521739131</v>
       </c>
     </row>
     <row r="10">
@@ -882,7 +882,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>4321288935.560001</v>
+        <v>4379404303.27</v>
       </c>
       <c r="C10" s="14" t="n"/>
       <c r="D10" s="14" t="n"/>
@@ -909,7 +909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2363,6 +2363,31 @@
       </c>
       <c r="G58" s="5" t="n">
         <v>138636.62</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B59" s="15" t="inlineStr">
+        <is>
+          <t>Ago</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="n">
+        <v>58115367.70999998</v>
+      </c>
+      <c r="D59" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="9" t="n">
+        <v>55021345.66999998</v>
+      </c>
+      <c r="F59" s="9" t="n">
+        <v>3094022.04</v>
+      </c>
+      <c r="G59" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3913,16 +3938,16 @@
         </is>
       </c>
       <c r="C70" s="7" t="n">
-        <v>6</v>
+        <v>5.9388</v>
       </c>
       <c r="D70" s="7" t="n">
-        <v>6.6235</v>
+        <v>7.8191</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>8.535</v>
+        <v>8.4499</v>
       </c>
       <c r="F70" s="7" t="n">
-        <v>9.375</v>
+        <v>9.294499999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3939,7 +3964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1212"/>
+  <dimension ref="A1:N1273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -69353,6 +69378,3300 @@
         </is>
       </c>
     </row>
+    <row r="1213">
+      <c r="A1213" s="19" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B1213" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1213" s="20" t="n">
+        <v>1069</v>
+      </c>
+      <c r="D1213" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1213" s="21" t="n">
+        <v>100.000059</v>
+      </c>
+      <c r="F1213" s="21" t="n">
+        <v>8.1182</v>
+      </c>
+      <c r="G1213" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1213" s="22" t="n">
+        <v>59000</v>
+      </c>
+      <c r="I1213" s="22" t="n">
+        <v>59000.03</v>
+      </c>
+      <c r="J1213" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1213" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1213" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1213" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1213" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="23" t="n">
+        <v>46238</v>
+      </c>
+      <c r="B1214" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1214" s="24" t="n">
+        <v>1069</v>
+      </c>
+      <c r="D1214" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1214" s="25" t="n">
+        <v>100.000059</v>
+      </c>
+      <c r="F1214" s="25" t="n">
+        <v>8.1182</v>
+      </c>
+      <c r="G1214" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1214" s="26" t="n">
+        <v>498550</v>
+      </c>
+      <c r="I1214" s="26" t="n">
+        <v>498550.29</v>
+      </c>
+      <c r="J1214" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1214" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1214" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1214" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1214" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="19" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B1215" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1215" s="20" t="n">
+        <v>1794</v>
+      </c>
+      <c r="D1215" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1215" s="21" t="n">
+        <v>100.000116</v>
+      </c>
+      <c r="F1215" s="21" t="n">
+        <v>8.289300000000001</v>
+      </c>
+      <c r="G1215" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1215" s="22" t="n">
+        <v>42000</v>
+      </c>
+      <c r="I1215" s="22" t="n">
+        <v>42000.05</v>
+      </c>
+      <c r="J1215" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1215" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1215" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1215" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1215" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="23" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B1216" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1216" s="24" t="n">
+        <v>1068</v>
+      </c>
+      <c r="D1216" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1216" s="25" t="n">
+        <v>100.000184</v>
+      </c>
+      <c r="F1216" s="25" t="n">
+        <v>8.118</v>
+      </c>
+      <c r="G1216" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1216" s="26" t="n">
+        <v>14000</v>
+      </c>
+      <c r="I1216" s="26" t="n">
+        <v>14000.03</v>
+      </c>
+      <c r="J1216" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1216" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1216" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1216" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1216" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="19" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B1217" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1217" s="20" t="n">
+        <v>1067</v>
+      </c>
+      <c r="D1217" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1217" s="21" t="n">
+        <v>100.000054</v>
+      </c>
+      <c r="F1217" s="21" t="n">
+        <v>8.117900000000001</v>
+      </c>
+      <c r="G1217" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1217" s="22" t="n">
+        <v>142100</v>
+      </c>
+      <c r="I1217" s="22" t="n">
+        <v>142100.08</v>
+      </c>
+      <c r="J1217" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1217" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1217" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1217" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1217" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="23" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B1218" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1218" s="24" t="n">
+        <v>1067</v>
+      </c>
+      <c r="D1218" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1218" s="25" t="n">
+        <v>100.000054</v>
+      </c>
+      <c r="F1218" s="25" t="n">
+        <v>8.117900000000001</v>
+      </c>
+      <c r="G1218" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1218" s="26" t="n">
+        <v>50300</v>
+      </c>
+      <c r="I1218" s="26" t="n">
+        <v>50300.03</v>
+      </c>
+      <c r="J1218" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1218" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1218" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1218" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1218" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="19" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B1219" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1219" s="20" t="n">
+        <v>1067</v>
+      </c>
+      <c r="D1219" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1219" s="21" t="n">
+        <v>100.000054</v>
+      </c>
+      <c r="F1219" s="21" t="n">
+        <v>8.117900000000001</v>
+      </c>
+      <c r="G1219" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1219" s="22" t="n">
+        <v>213894</v>
+      </c>
+      <c r="I1219" s="22" t="n">
+        <v>213894.12</v>
+      </c>
+      <c r="J1219" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1219" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1219" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1219" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1219" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="23" t="n">
+        <v>46240</v>
+      </c>
+      <c r="B1220" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1220" s="24" t="n">
+        <v>1793</v>
+      </c>
+      <c r="D1220" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1220" s="25" t="n">
+        <v>100.000085</v>
+      </c>
+      <c r="F1220" s="25" t="n">
+        <v>8.289199999999999</v>
+      </c>
+      <c r="G1220" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1220" s="26" t="n">
+        <v>212019</v>
+      </c>
+      <c r="I1220" s="26" t="n">
+        <v>212019.18</v>
+      </c>
+      <c r="J1220" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1220" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1220" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1220" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1220" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" s="19" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B1221" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1221" s="20" t="n">
+        <v>1066</v>
+      </c>
+      <c r="D1221" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1221" s="21" t="n">
+        <v>100.000187</v>
+      </c>
+      <c r="F1221" s="21" t="n">
+        <v>8.117699999999999</v>
+      </c>
+      <c r="G1221" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1221" s="22" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="I1221" s="22" t="n">
+        <v>4000007.48</v>
+      </c>
+      <c r="J1221" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1221" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1221" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1221" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1221" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" s="23" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B1222" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1222" s="24" t="n">
+        <v>1066</v>
+      </c>
+      <c r="D1222" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1222" s="25" t="n">
+        <v>100.000187</v>
+      </c>
+      <c r="F1222" s="25" t="n">
+        <v>8.117699999999999</v>
+      </c>
+      <c r="G1222" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1222" s="26" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="I1222" s="26" t="n">
+        <v>2500004.68</v>
+      </c>
+      <c r="J1222" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1222" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1222" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1222" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1222" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" s="19" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B1223" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1223" s="20" t="n">
+        <v>1066</v>
+      </c>
+      <c r="D1223" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1223" s="21" t="n">
+        <v>100.000187</v>
+      </c>
+      <c r="F1223" s="21" t="n">
+        <v>8.117699999999999</v>
+      </c>
+      <c r="G1223" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1223" s="22" t="n">
+        <v>500000</v>
+      </c>
+      <c r="I1223" s="22" t="n">
+        <v>500000.94</v>
+      </c>
+      <c r="J1223" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1223" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1223" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1223" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1223" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" s="23" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B1224" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1224" s="24" t="n">
+        <v>1066</v>
+      </c>
+      <c r="D1224" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1224" s="25" t="n">
+        <v>100.000187</v>
+      </c>
+      <c r="F1224" s="25" t="n">
+        <v>8.117699999999999</v>
+      </c>
+      <c r="G1224" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1224" s="26" t="n">
+        <v>900000</v>
+      </c>
+      <c r="I1224" s="26" t="n">
+        <v>900001.6800000001</v>
+      </c>
+      <c r="J1224" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1224" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1224" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1224" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1224" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" s="19" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B1225" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1225" s="20" t="n">
+        <v>1792</v>
+      </c>
+      <c r="D1225" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1225" s="21" t="n">
+        <v>100.000058</v>
+      </c>
+      <c r="F1225" s="21" t="n">
+        <v>8.289099999999999</v>
+      </c>
+      <c r="G1225" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1225" s="22" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1225" s="22" t="n">
+        <v>30000.02</v>
+      </c>
+      <c r="J1225" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1225" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1225" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1225" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1225" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" s="23" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B1226" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1226" s="24" t="n">
+        <v>1066</v>
+      </c>
+      <c r="D1226" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1226" s="25" t="n">
+        <v>100.000187</v>
+      </c>
+      <c r="F1226" s="25" t="n">
+        <v>8.117699999999999</v>
+      </c>
+      <c r="G1226" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1226" s="26" t="n">
+        <v>99641</v>
+      </c>
+      <c r="I1226" s="26" t="n">
+        <v>99641.19</v>
+      </c>
+      <c r="J1226" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1226" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1226" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1226" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1226" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" s="19" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B1227" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1227" s="20" t="n">
+        <v>1062</v>
+      </c>
+      <c r="D1227" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1227" s="21" t="n">
+        <v>100.000245</v>
+      </c>
+      <c r="F1227" s="21" t="n">
+        <v>8.117100000000001</v>
+      </c>
+      <c r="G1227" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1227" s="22" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I1227" s="22" t="n">
+        <v>40000.1</v>
+      </c>
+      <c r="J1227" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1227" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1227" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1227" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1227" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" s="23" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B1228" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1228" s="24" t="n">
+        <v>1062</v>
+      </c>
+      <c r="D1228" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1228" s="25" t="n">
+        <v>100.000245</v>
+      </c>
+      <c r="F1228" s="25" t="n">
+        <v>8.117100000000001</v>
+      </c>
+      <c r="G1228" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1228" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1228" s="26" t="n">
+        <v>50000.12</v>
+      </c>
+      <c r="J1228" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1228" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1228" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1228" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1228" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" s="19" t="n">
+        <v>46245</v>
+      </c>
+      <c r="B1229" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1229" s="20" t="n">
+        <v>1062</v>
+      </c>
+      <c r="D1229" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1229" s="21" t="n">
+        <v>100.000245</v>
+      </c>
+      <c r="F1229" s="21" t="n">
+        <v>8.117100000000001</v>
+      </c>
+      <c r="G1229" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1229" s="22" t="n">
+        <v>38000</v>
+      </c>
+      <c r="I1229" s="22" t="n">
+        <v>38000.09</v>
+      </c>
+      <c r="J1229" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1229" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1229" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1229" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1229" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1230" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1230" s="24" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1230" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1230" s="25" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1230" s="25" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1230" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1230" s="26" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="I1230" s="26" t="n">
+        <v>2100002.96</v>
+      </c>
+      <c r="J1230" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1230" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1230" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1230" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1230" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1231" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1231" s="20" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1231" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1231" s="21" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1231" s="21" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1231" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1231" s="22" t="n">
+        <v>497645</v>
+      </c>
+      <c r="I1231" s="22" t="n">
+        <v>497645.7</v>
+      </c>
+      <c r="J1231" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1231" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1231" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1231" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1231" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1232" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1232" s="24" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1232" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1232" s="25" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1232" s="25" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1232" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1232" s="26" t="n">
+        <v>696700</v>
+      </c>
+      <c r="I1232" s="26" t="n">
+        <v>696700.98</v>
+      </c>
+      <c r="J1232" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1232" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1232" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1232" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1232" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1233" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1233" s="20" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1233" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1233" s="21" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1233" s="21" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1233" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1233" s="22" t="n">
+        <v>26000</v>
+      </c>
+      <c r="I1233" s="22" t="n">
+        <v>26000.04</v>
+      </c>
+      <c r="J1233" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1233" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1233" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1233" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1233" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1234" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1234" s="24" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1234" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1234" s="25" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1234" s="25" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1234" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1234" s="26" t="n">
+        <v>62000</v>
+      </c>
+      <c r="I1234" s="26" t="n">
+        <v>62000.09</v>
+      </c>
+      <c r="J1234" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1234" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1234" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1234" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1234" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1235" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1235" s="20" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1235" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1235" s="21" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1235" s="21" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1235" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1235" s="22" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1235" s="22" t="n">
+        <v>20000.03</v>
+      </c>
+      <c r="J1235" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1235" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1235" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1235" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1235" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1236" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1236" s="24" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1236" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1236" s="25" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1236" s="25" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1236" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1236" s="26" t="n">
+        <v>22000</v>
+      </c>
+      <c r="I1236" s="26" t="n">
+        <v>22000.03</v>
+      </c>
+      <c r="J1236" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1236" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1236" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1236" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1236" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" s="19" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1237" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1237" s="20" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1237" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1237" s="21" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1237" s="21" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1237" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1237" s="22" t="n">
+        <v>22000</v>
+      </c>
+      <c r="I1237" s="22" t="n">
+        <v>22000.03</v>
+      </c>
+      <c r="J1237" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1237" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1237" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1237" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1237" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="B1238" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1238" s="24" t="n">
+        <v>1061</v>
+      </c>
+      <c r="D1238" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1238" s="25" t="n">
+        <v>100.000141</v>
+      </c>
+      <c r="F1238" s="25" t="n">
+        <v>8.117000000000001</v>
+      </c>
+      <c r="G1238" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1238" s="26" t="n">
+        <v>34000</v>
+      </c>
+      <c r="I1238" s="26" t="n">
+        <v>34000.05</v>
+      </c>
+      <c r="J1238" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1238" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1238" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1238" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1238" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" s="19" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B1239" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1239" s="20" t="n">
+        <v>940</v>
+      </c>
+      <c r="D1239" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1239" s="21" t="n">
+        <v>100.000094</v>
+      </c>
+      <c r="F1239" s="21" t="n">
+        <v>8.113899999999999</v>
+      </c>
+      <c r="G1239" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1239" s="22" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1239" s="22" t="n">
+        <v>1000000.94</v>
+      </c>
+      <c r="J1239" s="19" t="n">
+        <v>46104</v>
+      </c>
+      <c r="K1239" s="19" t="n">
+        <v>47200</v>
+      </c>
+      <c r="L1239" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1239" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1239" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" s="23" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B1240" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1240" s="24" t="n">
+        <v>948</v>
+      </c>
+      <c r="D1240" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1240" s="25" t="n">
+        <v>100.000003</v>
+      </c>
+      <c r="F1240" s="25" t="n">
+        <v>8.113200000000001</v>
+      </c>
+      <c r="G1240" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1240" s="26" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="I1240" s="26" t="n">
+        <v>2000000.05</v>
+      </c>
+      <c r="J1240" s="23" t="n">
+        <v>46113</v>
+      </c>
+      <c r="K1240" s="23" t="n">
+        <v>47209</v>
+      </c>
+      <c r="L1240" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1240" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1240" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" s="19" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B1241" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1241" s="20" t="n">
+        <v>1060</v>
+      </c>
+      <c r="D1241" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1241" s="21" t="n">
+        <v>100.000042</v>
+      </c>
+      <c r="F1241" s="21" t="n">
+        <v>8.116899999999999</v>
+      </c>
+      <c r="G1241" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1241" s="22" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="I1241" s="22" t="n">
+        <v>2000000.83</v>
+      </c>
+      <c r="J1241" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1241" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1241" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1241" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1241" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" s="23" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B1242" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1242" s="24" t="n">
+        <v>1060</v>
+      </c>
+      <c r="D1242" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1242" s="25" t="n">
+        <v>100.000042</v>
+      </c>
+      <c r="F1242" s="25" t="n">
+        <v>8.116899999999999</v>
+      </c>
+      <c r="G1242" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1242" s="26" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="I1242" s="26" t="n">
+        <v>6000002.5</v>
+      </c>
+      <c r="J1242" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1242" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1242" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1242" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1242" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" s="19" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B1243" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1243" s="20" t="n">
+        <v>1060</v>
+      </c>
+      <c r="D1243" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1243" s="21" t="n">
+        <v>100.000042</v>
+      </c>
+      <c r="F1243" s="21" t="n">
+        <v>8.116899999999999</v>
+      </c>
+      <c r="G1243" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1243" s="22" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="I1243" s="22" t="n">
+        <v>10000004.17</v>
+      </c>
+      <c r="J1243" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1243" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1243" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1243" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1243" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" s="23" t="n">
+        <v>46247</v>
+      </c>
+      <c r="B1244" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1244" s="24" t="n">
+        <v>1060</v>
+      </c>
+      <c r="D1244" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1244" s="25" t="n">
+        <v>100.000042</v>
+      </c>
+      <c r="F1244" s="25" t="n">
+        <v>8.116899999999999</v>
+      </c>
+      <c r="G1244" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1244" s="26" t="n">
+        <v>199500</v>
+      </c>
+      <c r="I1244" s="26" t="n">
+        <v>199500.08</v>
+      </c>
+      <c r="J1244" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1244" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1244" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1244" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1244" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" s="19" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B1245" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1245" s="20" t="n">
+        <v>1059</v>
+      </c>
+      <c r="D1245" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1245" s="21" t="n">
+        <v>100.000204</v>
+      </c>
+      <c r="F1245" s="21" t="n">
+        <v>8.1167</v>
+      </c>
+      <c r="G1245" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1245" s="22" t="n">
+        <v>80000</v>
+      </c>
+      <c r="I1245" s="22" t="n">
+        <v>80000.16</v>
+      </c>
+      <c r="J1245" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1245" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1245" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1245" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1245" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" s="23" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B1246" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1246" s="24" t="n">
+        <v>1785</v>
+      </c>
+      <c r="D1246" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1246" s="25" t="n">
+        <v>100.000006</v>
+      </c>
+      <c r="F1246" s="25" t="n">
+        <v>8.288399999999999</v>
+      </c>
+      <c r="G1246" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1246" s="26" t="n">
+        <v>300000</v>
+      </c>
+      <c r="I1246" s="26" t="n">
+        <v>300000.02</v>
+      </c>
+      <c r="J1246" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1246" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1246" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1246" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1246" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" s="19" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B1247" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1247" s="20" t="n">
+        <v>1059</v>
+      </c>
+      <c r="D1247" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1247" s="21" t="n">
+        <v>100.000204</v>
+      </c>
+      <c r="F1247" s="21" t="n">
+        <v>8.1167</v>
+      </c>
+      <c r="G1247" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1247" s="22" t="n">
+        <v>44000</v>
+      </c>
+      <c r="I1247" s="22" t="n">
+        <v>44000.09</v>
+      </c>
+      <c r="J1247" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1247" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1247" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1247" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1247" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" s="23" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B1248" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1248" s="24" t="n">
+        <v>1056</v>
+      </c>
+      <c r="D1248" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1248" s="25" t="n">
+        <v>100.000203</v>
+      </c>
+      <c r="F1248" s="25" t="n">
+        <v>8.116300000000001</v>
+      </c>
+      <c r="G1248" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1248" s="26" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I1248" s="26" t="n">
+        <v>5000.01</v>
+      </c>
+      <c r="J1248" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1248" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1248" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1248" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1248" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" s="19" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B1249" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1249" s="20" t="n">
+        <v>1056</v>
+      </c>
+      <c r="D1249" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1249" s="21" t="n">
+        <v>100.000203</v>
+      </c>
+      <c r="F1249" s="21" t="n">
+        <v>8.116300000000001</v>
+      </c>
+      <c r="G1249" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1249" s="22" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1249" s="22" t="n">
+        <v>10000.02</v>
+      </c>
+      <c r="J1249" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1249" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1249" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1249" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1249" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" s="23" t="n">
+        <v>46251</v>
+      </c>
+      <c r="B1250" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1250" s="24" t="n">
+        <v>1056</v>
+      </c>
+      <c r="D1250" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1250" s="25" t="n">
+        <v>100.000203</v>
+      </c>
+      <c r="F1250" s="25" t="n">
+        <v>8.116300000000001</v>
+      </c>
+      <c r="G1250" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1250" s="26" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I1250" s="26" t="n">
+        <v>7000.01</v>
+      </c>
+      <c r="J1250" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1250" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1250" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1250" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1250" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" s="19" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B1251" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1251" s="20" t="n">
+        <v>1055</v>
+      </c>
+      <c r="D1251" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1251" s="21" t="n">
+        <v>100.000126</v>
+      </c>
+      <c r="F1251" s="21" t="n">
+        <v>8.116199999999999</v>
+      </c>
+      <c r="G1251" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1251" s="22" t="n">
+        <v>22000</v>
+      </c>
+      <c r="I1251" s="22" t="n">
+        <v>22000.03</v>
+      </c>
+      <c r="J1251" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1251" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1251" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1251" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1251" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" s="23" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B1252" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1252" s="24" t="n">
+        <v>1055</v>
+      </c>
+      <c r="D1252" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1252" s="25" t="n">
+        <v>100.000126</v>
+      </c>
+      <c r="F1252" s="25" t="n">
+        <v>8.116199999999999</v>
+      </c>
+      <c r="G1252" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1252" s="26" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="I1252" s="26" t="n">
+        <v>1000001.26</v>
+      </c>
+      <c r="J1252" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1252" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1252" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1252" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1252" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" s="19" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B1253" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1253" s="20" t="n">
+        <v>1780</v>
+      </c>
+      <c r="D1253" s="15" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1253" s="21" t="n">
+        <v>100.000112</v>
+      </c>
+      <c r="F1253" s="21" t="n">
+        <v>8.2879</v>
+      </c>
+      <c r="G1253" s="21" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1253" s="22" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="I1253" s="22" t="n">
+        <v>2500002.8</v>
+      </c>
+      <c r="J1253" s="19" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1253" s="19" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1253" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1253" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1253" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" s="23" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B1254" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1254" s="24" t="n">
+        <v>1055</v>
+      </c>
+      <c r="D1254" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1254" s="25" t="n">
+        <v>100.000126</v>
+      </c>
+      <c r="F1254" s="25" t="n">
+        <v>8.116199999999999</v>
+      </c>
+      <c r="G1254" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1254" s="26" t="n">
+        <v>496975</v>
+      </c>
+      <c r="I1254" s="26" t="n">
+        <v>496975.62</v>
+      </c>
+      <c r="J1254" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1254" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1254" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1254" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1254" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" s="19" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B1255" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1255" s="20" t="n">
+        <v>1055</v>
+      </c>
+      <c r="D1255" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1255" s="21" t="n">
+        <v>100.000126</v>
+      </c>
+      <c r="F1255" s="21" t="n">
+        <v>8.116199999999999</v>
+      </c>
+      <c r="G1255" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1255" s="22" t="n">
+        <v>496975</v>
+      </c>
+      <c r="I1255" s="22" t="n">
+        <v>496975.62</v>
+      </c>
+      <c r="J1255" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1255" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1255" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1255" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1255" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" s="23" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B1256" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1256" s="24" t="n">
+        <v>1055</v>
+      </c>
+      <c r="D1256" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1256" s="25" t="n">
+        <v>100.000126</v>
+      </c>
+      <c r="F1256" s="25" t="n">
+        <v>8.116199999999999</v>
+      </c>
+      <c r="G1256" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1256" s="26" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="I1256" s="26" t="n">
+        <v>5000006.28</v>
+      </c>
+      <c r="J1256" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1256" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1256" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1256" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1256" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" s="19" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B1257" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1257" s="20" t="n">
+        <v>1054</v>
+      </c>
+      <c r="D1257" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1257" s="21" t="n">
+        <v>100.000053</v>
+      </c>
+      <c r="F1257" s="21" t="n">
+        <v>8.116099999999999</v>
+      </c>
+      <c r="G1257" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1257" s="22" t="n">
+        <v>50000</v>
+      </c>
+      <c r="I1257" s="22" t="n">
+        <v>50000.03</v>
+      </c>
+      <c r="J1257" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1257" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1257" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1257" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1257" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" s="23" t="n">
+        <v>46253</v>
+      </c>
+      <c r="B1258" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1258" s="24" t="n">
+        <v>1054</v>
+      </c>
+      <c r="D1258" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1258" s="25" t="n">
+        <v>100.000053</v>
+      </c>
+      <c r="F1258" s="25" t="n">
+        <v>8.116099999999999</v>
+      </c>
+      <c r="G1258" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1258" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1258" s="26" t="n">
+        <v>10000.01</v>
+      </c>
+      <c r="J1258" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1258" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1258" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1258" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1258" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1259" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1259" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1259" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1259" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1259" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1259" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1259" s="22" t="n">
+        <v>17000</v>
+      </c>
+      <c r="I1259" s="22" t="n">
+        <v>17000.04</v>
+      </c>
+      <c r="J1259" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1259" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1259" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1259" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1259" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" s="23" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1260" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1260" s="24" t="n">
+        <v>933</v>
+      </c>
+      <c r="D1260" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1260" s="25" t="n">
+        <v>100.000029</v>
+      </c>
+      <c r="F1260" s="25" t="n">
+        <v>8.114699999999999</v>
+      </c>
+      <c r="G1260" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1260" s="26" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="I1260" s="26" t="n">
+        <v>4000001.15</v>
+      </c>
+      <c r="J1260" s="23" t="n">
+        <v>46104</v>
+      </c>
+      <c r="K1260" s="23" t="n">
+        <v>47200</v>
+      </c>
+      <c r="L1260" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1260" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1260" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1261" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1261" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1261" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1261" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1261" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1261" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1261" s="22" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="I1261" s="22" t="n">
+        <v>8000019.24</v>
+      </c>
+      <c r="J1261" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1261" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1261" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1261" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1261" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1262">
+      <c r="A1262" s="23" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1262" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1262" s="24" t="n">
+        <v>1779</v>
+      </c>
+      <c r="D1262" s="16" t="inlineStr">
+        <is>
+          <t>De 3 a 5</t>
+        </is>
+      </c>
+      <c r="E1262" s="25" t="n">
+        <v>99.999748</v>
+      </c>
+      <c r="F1262" s="25" t="n">
+        <v>8.2879</v>
+      </c>
+      <c r="G1262" s="25" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="H1262" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I1262" s="26" t="n">
+        <v>9999.969999999999</v>
+      </c>
+      <c r="J1262" s="23" t="n">
+        <v>46232</v>
+      </c>
+      <c r="K1262" s="23" t="n">
+        <v>48058</v>
+      </c>
+      <c r="L1262" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1262" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1262" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1263" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1263" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1263" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1263" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1263" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1263" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1263" s="22" t="n">
+        <v>496800</v>
+      </c>
+      <c r="I1263" s="22" t="n">
+        <v>496801.19</v>
+      </c>
+      <c r="J1263" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1263" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1263" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1263" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1263" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" s="23" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1264" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1264" s="24" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1264" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1264" s="25" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1264" s="25" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1264" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1264" s="26" t="n">
+        <v>99400</v>
+      </c>
+      <c r="I1264" s="26" t="n">
+        <v>99400.24000000001</v>
+      </c>
+      <c r="J1264" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1264" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1264" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1264" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1264" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1265" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1265" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1265" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1265" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1265" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1265" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1265" s="22" t="n">
+        <v>993502</v>
+      </c>
+      <c r="I1265" s="22" t="n">
+        <v>993504.39</v>
+      </c>
+      <c r="J1265" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1265" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1265" s="15" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1265" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1265" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" s="23" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1266" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1266" s="24" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1266" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1266" s="25" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1266" s="25" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1266" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1266" s="26" t="n">
+        <v>42600</v>
+      </c>
+      <c r="I1266" s="26" t="n">
+        <v>42600.1</v>
+      </c>
+      <c r="J1266" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1266" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1266" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1266" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1266" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1267" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1267" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1267" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1267" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1267" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1267" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1267" s="22" t="n">
+        <v>5700</v>
+      </c>
+      <c r="I1267" s="22" t="n">
+        <v>5700.01</v>
+      </c>
+      <c r="J1267" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1267" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1267" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1267" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1267" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" s="23" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1268" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1268" s="24" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1268" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1268" s="25" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1268" s="25" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1268" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1268" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1268" s="26" t="n">
+        <v>30000.07</v>
+      </c>
+      <c r="J1268" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1268" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1268" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1268" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1268" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1269" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1269" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1269" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1269" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1269" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1269" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1269" s="22" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I1269" s="22" t="n">
+        <v>200000.48</v>
+      </c>
+      <c r="J1269" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1269" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1269" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1269" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1269" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" s="23" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1270" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1270" s="24" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1270" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1270" s="25" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1270" s="25" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1270" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1270" s="26" t="n">
+        <v>64000</v>
+      </c>
+      <c r="I1270" s="26" t="n">
+        <v>64000.15</v>
+      </c>
+      <c r="J1270" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1270" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1270" s="16" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1270" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1270" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" s="19" t="n">
+        <v>46254</v>
+      </c>
+      <c r="B1271" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1271" s="20" t="n">
+        <v>1053</v>
+      </c>
+      <c r="D1271" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1271" s="21" t="n">
+        <v>100.00024</v>
+      </c>
+      <c r="F1271" s="21" t="n">
+        <v>8.1159</v>
+      </c>
+      <c r="G1271" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1271" s="22" t="n">
+        <v>20000</v>
+      </c>
+      <c r="I1271" s="22" t="n">
+        <v>20000.05</v>
+      </c>
+      <c r="J1271" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1271" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1271" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1271" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1271" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" s="23" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B1272" s="16" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1272" s="24" t="n">
+        <v>1052</v>
+      </c>
+      <c r="D1272" s="16" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1272" s="25" t="n">
+        <v>100.000176</v>
+      </c>
+      <c r="F1272" s="25" t="n">
+        <v>8.1158</v>
+      </c>
+      <c r="G1272" s="25" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1272" s="26" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I1272" s="26" t="n">
+        <v>30000.05</v>
+      </c>
+      <c r="J1272" s="23" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1272" s="23" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1272" s="16" t="inlineStr">
+        <is>
+          <t>Q</t>
+        </is>
+      </c>
+      <c r="M1272" s="16" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1272" s="16" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" s="19" t="n">
+        <v>46255</v>
+      </c>
+      <c r="B1273" s="15" t="inlineStr">
+        <is>
+          <t>2026-005</t>
+        </is>
+      </c>
+      <c r="C1273" s="20" t="n">
+        <v>1052</v>
+      </c>
+      <c r="D1273" s="15" t="inlineStr">
+        <is>
+          <t>De 1 a 3</t>
+        </is>
+      </c>
+      <c r="E1273" s="21" t="n">
+        <v>100.000176</v>
+      </c>
+      <c r="F1273" s="21" t="n">
+        <v>8.1158</v>
+      </c>
+      <c r="G1273" s="21" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="H1273" s="22" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I1273" s="22" t="n">
+        <v>15000.03</v>
+      </c>
+      <c r="J1273" s="19" t="n">
+        <v>46226</v>
+      </c>
+      <c r="K1273" s="19" t="n">
+        <v>47322</v>
+      </c>
+      <c r="L1273" s="15" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="M1273" s="15" t="inlineStr">
+        <is>
+          <t>UNIC</t>
+        </is>
+      </c>
+      <c r="N1273" s="15" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N1"/>

</xml_diff>